<commit_message>
Add monthly quote workbook for the Hosen program, start both at September
Hosen workbook: one sheet per month (Sep 2026 - Sep 2027) listing the
Wednesday meetings with a 1,300 base fee plus 100 per participant (1-7),
a status per meeting following the agreed cancellation terms, agreed vs.
actual attendance, and separate columns for farm-approved special projects.
The rehab instruction workbook now also includes September 2026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GcyaTAwk1vz9KMfGvL4b7o
</commit_message>
<xml_diff>
--- a/quotes/הצעת-מחיר-חודשית-חוות-רום.xlsx
+++ b/quotes/הצעת-מחיר-חודשית-חוות-רום.xlsx
@@ -10,32 +10,34 @@
   <sheets>
     <sheet name="הוראות" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="הגדרות" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="אוקטובר 2026" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="נובמבר 2026" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="דצמבר 2026" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="ינואר 2027" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="פברואר 2027" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="מרץ 2027" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="אפריל 2027" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="מאי 2027" sheetId="10" state="visible" r:id="rId12"/>
-    <sheet name="יוני 2027" sheetId="11" state="visible" r:id="rId13"/>
-    <sheet name="יולי 2027" sheetId="12" state="visible" r:id="rId14"/>
-    <sheet name="אוגוסט 2027" sheetId="13" state="visible" r:id="rId15"/>
-    <sheet name="ספטמבר 2027" sheetId="14" state="visible" r:id="rId16"/>
+    <sheet name="ספטמבר 2026" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="אוקטובר 2026" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="נובמבר 2026" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="דצמבר 2026" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="ינואר 2027" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="פברואר 2027" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="מרץ 2027" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="אפריל 2027" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="מאי 2027" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="יוני 2027" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="יולי 2027" sheetId="13" state="visible" r:id="rId15"/>
+    <sheet name="אוגוסט 2027" sheetId="14" state="visible" r:id="rId16"/>
+    <sheet name="ספטמבר 2027" sheetId="15" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="12" name="_xlnm.Print_Area" vbProcedure="false">'אוגוסט 2027'!$A$1:$I$36</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">'אוקטובר 2026'!$A$1:$I$36</definedName>
-    <definedName function="false" hidden="false" localSheetId="8" name="_xlnm.Print_Area" vbProcedure="false">'אפריל 2027'!$A$1:$I$36</definedName>
-    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">'דצמבר 2026'!$A$1:$I$36</definedName>
-    <definedName function="false" hidden="false" localSheetId="11" name="_xlnm.Print_Area" vbProcedure="false">'יולי 2027'!$A$1:$I$36</definedName>
-    <definedName function="false" hidden="false" localSheetId="10" name="_xlnm.Print_Area" vbProcedure="false">'יוני 2027'!$A$1:$I$36</definedName>
-    <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Area" vbProcedure="false">'ינואר 2027'!$A$1:$I$36</definedName>
-    <definedName function="false" hidden="false" localSheetId="9" name="_xlnm.Print_Area" vbProcedure="false">'מאי 2027'!$A$1:$I$36</definedName>
-    <definedName function="false" hidden="false" localSheetId="7" name="_xlnm.Print_Area" vbProcedure="false">'מרץ 2027'!$A$1:$I$36</definedName>
-    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">'נובמבר 2026'!$A$1:$I$36</definedName>
-    <definedName function="false" hidden="false" localSheetId="13" name="_xlnm.Print_Area" vbProcedure="false">'ספטמבר 2027'!$A$1:$I$36</definedName>
-    <definedName function="false" hidden="false" localSheetId="6" name="_xlnm.Print_Area" vbProcedure="false">'פברואר 2027'!$A$1:$I$36</definedName>
+    <definedName function="false" hidden="false" localSheetId="13" name="_xlnm.Print_Area" vbProcedure="false">'אוגוסט 2027'!$A$1:$I$36</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">'אוקטובר 2026'!$A$1:$I$36</definedName>
+    <definedName function="false" hidden="false" localSheetId="9" name="_xlnm.Print_Area" vbProcedure="false">'אפריל 2027'!$A$1:$I$36</definedName>
+    <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Area" vbProcedure="false">'דצמבר 2026'!$A$1:$I$36</definedName>
+    <definedName function="false" hidden="false" localSheetId="12" name="_xlnm.Print_Area" vbProcedure="false">'יולי 2027'!$A$1:$I$36</definedName>
+    <definedName function="false" hidden="false" localSheetId="11" name="_xlnm.Print_Area" vbProcedure="false">'יוני 2027'!$A$1:$I$36</definedName>
+    <definedName function="false" hidden="false" localSheetId="6" name="_xlnm.Print_Area" vbProcedure="false">'ינואר 2027'!$A$1:$I$36</definedName>
+    <definedName function="false" hidden="false" localSheetId="10" name="_xlnm.Print_Area" vbProcedure="false">'מאי 2027'!$A$1:$I$36</definedName>
+    <definedName function="false" hidden="false" localSheetId="8" name="_xlnm.Print_Area" vbProcedure="false">'מרץ 2027'!$A$1:$I$36</definedName>
+    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">'נובמבר 2026'!$A$1:$I$36</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">'ספטמבר 2026'!$A$1:$I$36</definedName>
+    <definedName function="false" hidden="false" localSheetId="14" name="_xlnm.Print_Area" vbProcedure="false">'ספטמבר 2027'!$A$1:$I$36</definedName>
+    <definedName function="false" hidden="false" localSheetId="7" name="_xlnm.Print_Area" vbProcedure="false">'פברואר 2027'!$A$1:$I$36</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -247,6 +249,56 @@
 </file>
 
 <file path=xl/comments14.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="B25" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="FreeSans"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">תאריך ישיבת הצוות – לא חובה</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="FreeSans"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">אפשר להקליד כל תאריך בחודש (למשל </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">1/11/2026) – כל התאריכים בטבלה מתעדכנים לפיו.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments15.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
     <author>Unknown Author</author>
@@ -753,7 +805,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="92">
   <si>
     <t xml:space="preserve">איך משתמשים בקובץ</t>
   </si>
@@ -767,7 +819,7 @@
     <t xml:space="preserve">2. בסוף כל חודש</t>
   </si>
   <si>
-    <t xml:space="preserve">פותחים את הגיליון של החודש (למשל "אוקטובר 2026"). התאריכים של ימי ראשון וחמישי בחודש מחושבים אוטומטית, וכך גם השעות והסכומים.</t>
+    <t xml:space="preserve">פותחים את הגיליון של החודש (למשל "ספטמבר 2026"). התאריכים של ימי ראשון וחמישי בחודש מחושבים אוטומטית, וכך גם השעות והסכומים.</t>
   </si>
   <si>
     <t xml:space="preserve">3. ימים שלא התקיימו</t>
@@ -2028,13 +2080,13 @@
       <c r="I1" s="26"/>
       <c r="K1" s="27" t="n">
         <f aca="false">DATE(YEAR($H$11),MONTH($H$11),1)</f>
-        <v>46508</v>
+        <v>46478</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="str">
         <f aca="false">הגדרות!$C$17&amp;" · "&amp;CHOOSE(MONTH($K$1),"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר")&amp;" "&amp;YEAR($K$1)</f>
-        <v>הדרכת שיקום · מאי 2027</v>
+        <v>הדרכת שיקום · אפריל 2027</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -2046,7 +2098,7 @@
       <c r="I2" s="28"/>
       <c r="K2" s="27" t="n">
         <f aca="false">EOMONTH($K$1,0)</f>
-        <v>46538</v>
+        <v>46507</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2154,7 +2206,7 @@
       <c r="B11" s="30"/>
       <c r="C11" s="31" t="str">
         <f aca="false">YEAR($K$1)&amp;"-"&amp;TEXT(MONTH($K$1),"00")</f>
-        <v>2027-05</v>
+        <v>2027-04</v>
       </c>
       <c r="D11" s="31"/>
       <c r="F11" s="30" t="s">
@@ -2162,7 +2214,7 @@
       </c>
       <c r="G11" s="30"/>
       <c r="H11" s="32" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="I11" s="32"/>
     </row>
@@ -2173,7 +2225,7 @@
       <c r="B12" s="30"/>
       <c r="C12" s="33" t="n">
         <f aca="false">$K$2</f>
-        <v>46538</v>
+        <v>46507</v>
       </c>
       <c r="D12" s="33"/>
       <c r="F12" s="30" t="s">
@@ -2237,11 +2289,11 @@
       </c>
       <c r="B15" s="39" t="n">
         <f aca="false">$K$1+MIN(MOD(הגדרות!$D$18-WEEKDAY($K$1),7),MOD(הגדרות!$D$19-WEEKDAY($K$1),7))</f>
-        <v>46509</v>
+        <v>46478</v>
       </c>
       <c r="C15" s="38" t="str">
         <f aca="false">IF(B15="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B15)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D15" s="40" t="str">
         <f aca="false">IF(B15="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -2262,7 +2314,7 @@
       <c r="I15" s="45"/>
       <c r="K15" s="27" t="n">
         <f aca="false">IF(B15="","",B15+MIN(MOD(הגדרות!$D$18-WEEKDAY(B15)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B15)-1,7)+1))</f>
-        <v>46513</v>
+        <v>46481</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2272,11 +2324,11 @@
       </c>
       <c r="B16" s="39" t="n">
         <f aca="false">IF(K15="","",IF(K15&gt;$K$2,"",K15))</f>
-        <v>46513</v>
+        <v>46481</v>
       </c>
       <c r="C16" s="38" t="str">
         <f aca="false">IF(B16="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B16)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D16" s="40" t="str">
         <f aca="false">IF(B16="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -2297,7 +2349,7 @@
       <c r="I16" s="45"/>
       <c r="K16" s="27" t="n">
         <f aca="false">IF(B16="","",B16+MIN(MOD(הגדרות!$D$18-WEEKDAY(B16)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B16)-1,7)+1))</f>
-        <v>46516</v>
+        <v>46485</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2307,11 +2359,11 @@
       </c>
       <c r="B17" s="39" t="n">
         <f aca="false">IF(K16="","",IF(K16&gt;$K$2,"",K16))</f>
-        <v>46516</v>
+        <v>46485</v>
       </c>
       <c r="C17" s="38" t="str">
         <f aca="false">IF(B17="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B17)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D17" s="40" t="str">
         <f aca="false">IF(B17="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -2332,7 +2384,7 @@
       <c r="I17" s="45"/>
       <c r="K17" s="27" t="n">
         <f aca="false">IF(B17="","",B17+MIN(MOD(הגדרות!$D$18-WEEKDAY(B17)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B17)-1,7)+1))</f>
-        <v>46520</v>
+        <v>46488</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2342,11 +2394,11 @@
       </c>
       <c r="B18" s="39" t="n">
         <f aca="false">IF(K17="","",IF(K17&gt;$K$2,"",K17))</f>
-        <v>46520</v>
+        <v>46488</v>
       </c>
       <c r="C18" s="38" t="str">
         <f aca="false">IF(B18="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B18)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D18" s="40" t="str">
         <f aca="false">IF(B18="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -2367,7 +2419,7 @@
       <c r="I18" s="45"/>
       <c r="K18" s="27" t="n">
         <f aca="false">IF(B18="","",B18+MIN(MOD(הגדרות!$D$18-WEEKDAY(B18)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B18)-1,7)+1))</f>
-        <v>46523</v>
+        <v>46492</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2377,11 +2429,11 @@
       </c>
       <c r="B19" s="39" t="n">
         <f aca="false">IF(K18="","",IF(K18&gt;$K$2,"",K18))</f>
-        <v>46523</v>
+        <v>46492</v>
       </c>
       <c r="C19" s="38" t="str">
         <f aca="false">IF(B19="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B19)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D19" s="40" t="str">
         <f aca="false">IF(B19="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -2402,7 +2454,7 @@
       <c r="I19" s="45"/>
       <c r="K19" s="27" t="n">
         <f aca="false">IF(B19="","",B19+MIN(MOD(הגדרות!$D$18-WEEKDAY(B19)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B19)-1,7)+1))</f>
-        <v>46527</v>
+        <v>46495</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2412,11 +2464,11 @@
       </c>
       <c r="B20" s="39" t="n">
         <f aca="false">IF(K19="","",IF(K19&gt;$K$2,"",K19))</f>
-        <v>46527</v>
+        <v>46495</v>
       </c>
       <c r="C20" s="38" t="str">
         <f aca="false">IF(B20="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B20)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D20" s="40" t="str">
         <f aca="false">IF(B20="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -2437,7 +2489,7 @@
       <c r="I20" s="45"/>
       <c r="K20" s="27" t="n">
         <f aca="false">IF(B20="","",B20+MIN(MOD(הגדרות!$D$18-WEEKDAY(B20)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B20)-1,7)+1))</f>
-        <v>46530</v>
+        <v>46499</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2447,11 +2499,11 @@
       </c>
       <c r="B21" s="39" t="n">
         <f aca="false">IF(K20="","",IF(K20&gt;$K$2,"",K20))</f>
-        <v>46530</v>
+        <v>46499</v>
       </c>
       <c r="C21" s="38" t="str">
         <f aca="false">IF(B21="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B21)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D21" s="40" t="str">
         <f aca="false">IF(B21="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -2472,7 +2524,7 @@
       <c r="I21" s="45"/>
       <c r="K21" s="27" t="n">
         <f aca="false">IF(B21="","",B21+MIN(MOD(הגדרות!$D$18-WEEKDAY(B21)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B21)-1,7)+1))</f>
-        <v>46534</v>
+        <v>46502</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2482,11 +2534,11 @@
       </c>
       <c r="B22" s="39" t="n">
         <f aca="false">IF(K21="","",IF(K21&gt;$K$2,"",K21))</f>
-        <v>46534</v>
+        <v>46502</v>
       </c>
       <c r="C22" s="38" t="str">
         <f aca="false">IF(B22="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B22)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D22" s="40" t="str">
         <f aca="false">IF(B22="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -2507,7 +2559,7 @@
       <c r="I22" s="45"/>
       <c r="K22" s="27" t="n">
         <f aca="false">IF(B22="","",B22+MIN(MOD(הגדרות!$D$18-WEEKDAY(B22)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B22)-1,7)+1))</f>
-        <v>46537</v>
+        <v>46506</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2517,11 +2569,11 @@
       </c>
       <c r="B23" s="39" t="n">
         <f aca="false">IF(K22="","",IF(K22&gt;$K$2,"",K22))</f>
-        <v>46537</v>
+        <v>46506</v>
       </c>
       <c r="C23" s="38" t="str">
         <f aca="false">IF(B23="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B23)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D23" s="40" t="str">
         <f aca="false">IF(B23="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -2542,7 +2594,7 @@
       <c r="I23" s="45"/>
       <c r="K23" s="27" t="n">
         <f aca="false">IF(B23="","",B23+MIN(MOD(הגדרות!$D$18-WEEKDAY(B23)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B23)-1,7)+1))</f>
-        <v>46541</v>
+        <v>46509</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2859,13 +2911,13 @@
       <c r="I1" s="26"/>
       <c r="K1" s="27" t="n">
         <f aca="false">DATE(YEAR($H$11),MONTH($H$11),1)</f>
-        <v>46539</v>
+        <v>46508</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="str">
         <f aca="false">הגדרות!$C$17&amp;" · "&amp;CHOOSE(MONTH($K$1),"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר")&amp;" "&amp;YEAR($K$1)</f>
-        <v>הדרכת שיקום · יוני 2027</v>
+        <v>הדרכת שיקום · מאי 2027</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -2877,7 +2929,7 @@
       <c r="I2" s="28"/>
       <c r="K2" s="27" t="n">
         <f aca="false">EOMONTH($K$1,0)</f>
-        <v>46568</v>
+        <v>46538</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2985,7 +3037,7 @@
       <c r="B11" s="30"/>
       <c r="C11" s="31" t="str">
         <f aca="false">YEAR($K$1)&amp;"-"&amp;TEXT(MONTH($K$1),"00")</f>
-        <v>2027-06</v>
+        <v>2027-05</v>
       </c>
       <c r="D11" s="31"/>
       <c r="F11" s="30" t="s">
@@ -2993,7 +3045,7 @@
       </c>
       <c r="G11" s="30"/>
       <c r="H11" s="32" t="n">
-        <v>46539</v>
+        <v>46508</v>
       </c>
       <c r="I11" s="32"/>
     </row>
@@ -3004,7 +3056,7 @@
       <c r="B12" s="30"/>
       <c r="C12" s="33" t="n">
         <f aca="false">$K$2</f>
-        <v>46568</v>
+        <v>46538</v>
       </c>
       <c r="D12" s="33"/>
       <c r="F12" s="30" t="s">
@@ -3068,11 +3120,11 @@
       </c>
       <c r="B15" s="39" t="n">
         <f aca="false">$K$1+MIN(MOD(הגדרות!$D$18-WEEKDAY($K$1),7),MOD(הגדרות!$D$19-WEEKDAY($K$1),7))</f>
-        <v>46541</v>
+        <v>46509</v>
       </c>
       <c r="C15" s="38" t="str">
         <f aca="false">IF(B15="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B15)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D15" s="40" t="str">
         <f aca="false">IF(B15="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -3093,7 +3145,7 @@
       <c r="I15" s="45"/>
       <c r="K15" s="27" t="n">
         <f aca="false">IF(B15="","",B15+MIN(MOD(הגדרות!$D$18-WEEKDAY(B15)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B15)-1,7)+1))</f>
-        <v>46544</v>
+        <v>46513</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3103,11 +3155,11 @@
       </c>
       <c r="B16" s="39" t="n">
         <f aca="false">IF(K15="","",IF(K15&gt;$K$2,"",K15))</f>
-        <v>46544</v>
+        <v>46513</v>
       </c>
       <c r="C16" s="38" t="str">
         <f aca="false">IF(B16="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B16)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D16" s="40" t="str">
         <f aca="false">IF(B16="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -3128,7 +3180,7 @@
       <c r="I16" s="45"/>
       <c r="K16" s="27" t="n">
         <f aca="false">IF(B16="","",B16+MIN(MOD(הגדרות!$D$18-WEEKDAY(B16)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B16)-1,7)+1))</f>
-        <v>46548</v>
+        <v>46516</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3138,11 +3190,11 @@
       </c>
       <c r="B17" s="39" t="n">
         <f aca="false">IF(K16="","",IF(K16&gt;$K$2,"",K16))</f>
-        <v>46548</v>
+        <v>46516</v>
       </c>
       <c r="C17" s="38" t="str">
         <f aca="false">IF(B17="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B17)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D17" s="40" t="str">
         <f aca="false">IF(B17="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -3163,7 +3215,7 @@
       <c r="I17" s="45"/>
       <c r="K17" s="27" t="n">
         <f aca="false">IF(B17="","",B17+MIN(MOD(הגדרות!$D$18-WEEKDAY(B17)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B17)-1,7)+1))</f>
-        <v>46551</v>
+        <v>46520</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3173,11 +3225,11 @@
       </c>
       <c r="B18" s="39" t="n">
         <f aca="false">IF(K17="","",IF(K17&gt;$K$2,"",K17))</f>
-        <v>46551</v>
+        <v>46520</v>
       </c>
       <c r="C18" s="38" t="str">
         <f aca="false">IF(B18="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B18)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D18" s="40" t="str">
         <f aca="false">IF(B18="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -3198,7 +3250,7 @@
       <c r="I18" s="45"/>
       <c r="K18" s="27" t="n">
         <f aca="false">IF(B18="","",B18+MIN(MOD(הגדרות!$D$18-WEEKDAY(B18)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B18)-1,7)+1))</f>
-        <v>46555</v>
+        <v>46523</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3208,11 +3260,11 @@
       </c>
       <c r="B19" s="39" t="n">
         <f aca="false">IF(K18="","",IF(K18&gt;$K$2,"",K18))</f>
-        <v>46555</v>
+        <v>46523</v>
       </c>
       <c r="C19" s="38" t="str">
         <f aca="false">IF(B19="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B19)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D19" s="40" t="str">
         <f aca="false">IF(B19="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -3233,7 +3285,7 @@
       <c r="I19" s="45"/>
       <c r="K19" s="27" t="n">
         <f aca="false">IF(B19="","",B19+MIN(MOD(הגדרות!$D$18-WEEKDAY(B19)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B19)-1,7)+1))</f>
-        <v>46558</v>
+        <v>46527</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3243,11 +3295,11 @@
       </c>
       <c r="B20" s="39" t="n">
         <f aca="false">IF(K19="","",IF(K19&gt;$K$2,"",K19))</f>
-        <v>46558</v>
+        <v>46527</v>
       </c>
       <c r="C20" s="38" t="str">
         <f aca="false">IF(B20="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B20)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D20" s="40" t="str">
         <f aca="false">IF(B20="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -3268,7 +3320,7 @@
       <c r="I20" s="45"/>
       <c r="K20" s="27" t="n">
         <f aca="false">IF(B20="","",B20+MIN(MOD(הגדרות!$D$18-WEEKDAY(B20)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B20)-1,7)+1))</f>
-        <v>46562</v>
+        <v>46530</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3278,11 +3330,11 @@
       </c>
       <c r="B21" s="39" t="n">
         <f aca="false">IF(K20="","",IF(K20&gt;$K$2,"",K20))</f>
-        <v>46562</v>
+        <v>46530</v>
       </c>
       <c r="C21" s="38" t="str">
         <f aca="false">IF(B21="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B21)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D21" s="40" t="str">
         <f aca="false">IF(B21="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -3303,7 +3355,7 @@
       <c r="I21" s="45"/>
       <c r="K21" s="27" t="n">
         <f aca="false">IF(B21="","",B21+MIN(MOD(הגדרות!$D$18-WEEKDAY(B21)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B21)-1,7)+1))</f>
-        <v>46565</v>
+        <v>46534</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3313,11 +3365,11 @@
       </c>
       <c r="B22" s="39" t="n">
         <f aca="false">IF(K21="","",IF(K21&gt;$K$2,"",K21))</f>
-        <v>46565</v>
+        <v>46534</v>
       </c>
       <c r="C22" s="38" t="str">
         <f aca="false">IF(B22="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B22)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D22" s="40" t="str">
         <f aca="false">IF(B22="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -3338,42 +3390,42 @@
       <c r="I22" s="45"/>
       <c r="K22" s="27" t="n">
         <f aca="false">IF(B22="","",B22+MIN(MOD(הגדרות!$D$18-WEEKDAY(B22)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B22)-1,7)+1))</f>
-        <v>46569</v>
+        <v>46537</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="38" t="str">
+      <c r="A23" s="38" t="n">
         <f aca="false">IF(B23="","",ROW()-14)</f>
-        <v/>
-      </c>
-      <c r="B23" s="39" t="str">
+        <v>9</v>
+      </c>
+      <c r="B23" s="39" t="n">
         <f aca="false">IF(K22="","",IF(K22&gt;$K$2,"",K22))</f>
-        <v/>
+        <v>46537</v>
       </c>
       <c r="C23" s="38" t="str">
         <f aca="false">IF(B23="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B23)))</f>
-        <v/>
+        <v>ראשון</v>
       </c>
       <c r="D23" s="40" t="str">
         <f aca="false">IF(B23="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
-        <v/>
+        <v>הדרכה 09:00–12:30</v>
       </c>
       <c r="E23" s="41" t="s">
         <v>83</v>
       </c>
-      <c r="F23" s="42" t="str">
+      <c r="F23" s="42" t="n">
         <f aca="false">IF(B23="","",IF(E23="לא",0,הגדרות!$C$22))</f>
-        <v/>
-      </c>
-      <c r="G23" s="43" t="str">
+        <v>3.5</v>
+      </c>
+      <c r="G23" s="43" t="n">
         <f aca="false">IF(B23="","",F23*הגדרות!$C$24)</f>
-        <v/>
+        <v>175</v>
       </c>
       <c r="H23" s="44"/>
       <c r="I23" s="45"/>
-      <c r="K23" s="27" t="str">
+      <c r="K23" s="27" t="n">
         <f aca="false">IF(B23="","",B23+MIN(MOD(הגדרות!$D$18-WEEKDAY(B23)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B23)-1,7)+1))</f>
-        <v/>
+        <v>46541</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3414,7 +3466,7 @@
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="38" t="n">
         <f aca="false">COUNT($B$15:$B$24)+1</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B25" s="46"/>
       <c r="C25" s="38" t="str">
@@ -3449,11 +3501,11 @@
       <c r="E26" s="47"/>
       <c r="F26" s="48" t="n">
         <f aca="false">SUM(F15:F25)</f>
-        <v>29</v>
+        <v>32.5</v>
       </c>
       <c r="G26" s="49" t="n">
         <f aca="false">SUM(G15:G25)</f>
-        <v>1450</v>
+        <v>1625</v>
       </c>
       <c r="H26" s="47"/>
       <c r="I26" s="49" t="n">
@@ -3475,7 +3527,7 @@
       <c r="H28" s="40"/>
       <c r="I28" s="42" t="n">
         <f aca="false">F26</f>
-        <v>29</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3489,13 +3541,13 @@
       <c r="E29" s="51"/>
       <c r="F29" s="40" t="str">
         <f aca="false">"הדרכת שיקום ("&amp;TEXT(F26,"0.0")&amp;" שעות × "&amp;הגדרות!$C$24&amp;" ₪)"</f>
-        <v>הדרכת שיקום (29.0 שעות × 50 ₪)</v>
+        <v>הדרכת שיקום (32.5 שעות × 50 ₪)</v>
       </c>
       <c r="G29" s="40"/>
       <c r="H29" s="40"/>
       <c r="I29" s="43" t="n">
         <f aca="false">G26</f>
-        <v>1450</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3533,7 +3585,7 @@
       <c r="H31" s="52"/>
       <c r="I31" s="53" t="n">
         <f aca="false">I29+I30</f>
-        <v>1450</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3553,7 +3605,7 @@
       <c r="H32" s="40"/>
       <c r="I32" s="43" t="n">
         <f aca="false">ROUND(I31*הגדרות!$C$25,2)</f>
-        <v>261</v>
+        <v>292.5</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3564,7 +3616,7 @@
       <c r="H33" s="54"/>
       <c r="I33" s="55" t="n">
         <f aca="false">I31+I32</f>
-        <v>1711</v>
+        <v>1917.5</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3690,13 +3742,13 @@
       <c r="I1" s="26"/>
       <c r="K1" s="27" t="n">
         <f aca="false">DATE(YEAR($H$11),MONTH($H$11),1)</f>
-        <v>46569</v>
+        <v>46539</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="str">
         <f aca="false">הגדרות!$C$17&amp;" · "&amp;CHOOSE(MONTH($K$1),"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר")&amp;" "&amp;YEAR($K$1)</f>
-        <v>הדרכת שיקום · יולי 2027</v>
+        <v>הדרכת שיקום · יוני 2027</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -3708,7 +3760,7 @@
       <c r="I2" s="28"/>
       <c r="K2" s="27" t="n">
         <f aca="false">EOMONTH($K$1,0)</f>
-        <v>46599</v>
+        <v>46568</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3816,7 +3868,7 @@
       <c r="B11" s="30"/>
       <c r="C11" s="31" t="str">
         <f aca="false">YEAR($K$1)&amp;"-"&amp;TEXT(MONTH($K$1),"00")</f>
-        <v>2027-07</v>
+        <v>2027-06</v>
       </c>
       <c r="D11" s="31"/>
       <c r="F11" s="30" t="s">
@@ -3824,7 +3876,7 @@
       </c>
       <c r="G11" s="30"/>
       <c r="H11" s="32" t="n">
-        <v>46569</v>
+        <v>46539</v>
       </c>
       <c r="I11" s="32"/>
     </row>
@@ -3835,7 +3887,7 @@
       <c r="B12" s="30"/>
       <c r="C12" s="33" t="n">
         <f aca="false">$K$2</f>
-        <v>46599</v>
+        <v>46568</v>
       </c>
       <c r="D12" s="33"/>
       <c r="F12" s="30" t="s">
@@ -3899,7 +3951,7 @@
       </c>
       <c r="B15" s="39" t="n">
         <f aca="false">$K$1+MIN(MOD(הגדרות!$D$18-WEEKDAY($K$1),7),MOD(הגדרות!$D$19-WEEKDAY($K$1),7))</f>
-        <v>46569</v>
+        <v>46541</v>
       </c>
       <c r="C15" s="38" t="str">
         <f aca="false">IF(B15="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B15)))</f>
@@ -3924,7 +3976,7 @@
       <c r="I15" s="45"/>
       <c r="K15" s="27" t="n">
         <f aca="false">IF(B15="","",B15+MIN(MOD(הגדרות!$D$18-WEEKDAY(B15)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B15)-1,7)+1))</f>
-        <v>46572</v>
+        <v>46544</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3934,7 +3986,7 @@
       </c>
       <c r="B16" s="39" t="n">
         <f aca="false">IF(K15="","",IF(K15&gt;$K$2,"",K15))</f>
-        <v>46572</v>
+        <v>46544</v>
       </c>
       <c r="C16" s="38" t="str">
         <f aca="false">IF(B16="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B16)))</f>
@@ -3959,7 +4011,7 @@
       <c r="I16" s="45"/>
       <c r="K16" s="27" t="n">
         <f aca="false">IF(B16="","",B16+MIN(MOD(הגדרות!$D$18-WEEKDAY(B16)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B16)-1,7)+1))</f>
-        <v>46576</v>
+        <v>46548</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3969,7 +4021,7 @@
       </c>
       <c r="B17" s="39" t="n">
         <f aca="false">IF(K16="","",IF(K16&gt;$K$2,"",K16))</f>
-        <v>46576</v>
+        <v>46548</v>
       </c>
       <c r="C17" s="38" t="str">
         <f aca="false">IF(B17="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B17)))</f>
@@ -3994,7 +4046,7 @@
       <c r="I17" s="45"/>
       <c r="K17" s="27" t="n">
         <f aca="false">IF(B17="","",B17+MIN(MOD(הגדרות!$D$18-WEEKDAY(B17)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B17)-1,7)+1))</f>
-        <v>46579</v>
+        <v>46551</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4004,7 +4056,7 @@
       </c>
       <c r="B18" s="39" t="n">
         <f aca="false">IF(K17="","",IF(K17&gt;$K$2,"",K17))</f>
-        <v>46579</v>
+        <v>46551</v>
       </c>
       <c r="C18" s="38" t="str">
         <f aca="false">IF(B18="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B18)))</f>
@@ -4029,7 +4081,7 @@
       <c r="I18" s="45"/>
       <c r="K18" s="27" t="n">
         <f aca="false">IF(B18="","",B18+MIN(MOD(הגדרות!$D$18-WEEKDAY(B18)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B18)-1,7)+1))</f>
-        <v>46583</v>
+        <v>46555</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4039,7 +4091,7 @@
       </c>
       <c r="B19" s="39" t="n">
         <f aca="false">IF(K18="","",IF(K18&gt;$K$2,"",K18))</f>
-        <v>46583</v>
+        <v>46555</v>
       </c>
       <c r="C19" s="38" t="str">
         <f aca="false">IF(B19="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B19)))</f>
@@ -4064,7 +4116,7 @@
       <c r="I19" s="45"/>
       <c r="K19" s="27" t="n">
         <f aca="false">IF(B19="","",B19+MIN(MOD(הגדרות!$D$18-WEEKDAY(B19)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B19)-1,7)+1))</f>
-        <v>46586</v>
+        <v>46558</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4074,7 +4126,7 @@
       </c>
       <c r="B20" s="39" t="n">
         <f aca="false">IF(K19="","",IF(K19&gt;$K$2,"",K19))</f>
-        <v>46586</v>
+        <v>46558</v>
       </c>
       <c r="C20" s="38" t="str">
         <f aca="false">IF(B20="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B20)))</f>
@@ -4099,7 +4151,7 @@
       <c r="I20" s="45"/>
       <c r="K20" s="27" t="n">
         <f aca="false">IF(B20="","",B20+MIN(MOD(הגדרות!$D$18-WEEKDAY(B20)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B20)-1,7)+1))</f>
-        <v>46590</v>
+        <v>46562</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4109,7 +4161,7 @@
       </c>
       <c r="B21" s="39" t="n">
         <f aca="false">IF(K20="","",IF(K20&gt;$K$2,"",K20))</f>
-        <v>46590</v>
+        <v>46562</v>
       </c>
       <c r="C21" s="38" t="str">
         <f aca="false">IF(B21="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B21)))</f>
@@ -4134,7 +4186,7 @@
       <c r="I21" s="45"/>
       <c r="K21" s="27" t="n">
         <f aca="false">IF(B21="","",B21+MIN(MOD(הגדרות!$D$18-WEEKDAY(B21)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B21)-1,7)+1))</f>
-        <v>46593</v>
+        <v>46565</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4144,7 +4196,7 @@
       </c>
       <c r="B22" s="39" t="n">
         <f aca="false">IF(K21="","",IF(K21&gt;$K$2,"",K21))</f>
-        <v>46593</v>
+        <v>46565</v>
       </c>
       <c r="C22" s="38" t="str">
         <f aca="false">IF(B22="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B22)))</f>
@@ -4169,42 +4221,42 @@
       <c r="I22" s="45"/>
       <c r="K22" s="27" t="n">
         <f aca="false">IF(B22="","",B22+MIN(MOD(הגדרות!$D$18-WEEKDAY(B22)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B22)-1,7)+1))</f>
-        <v>46597</v>
+        <v>46569</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="38" t="n">
+      <c r="A23" s="38" t="str">
         <f aca="false">IF(B23="","",ROW()-14)</f>
-        <v>9</v>
-      </c>
-      <c r="B23" s="39" t="n">
+        <v/>
+      </c>
+      <c r="B23" s="39" t="str">
         <f aca="false">IF(K22="","",IF(K22&gt;$K$2,"",K22))</f>
-        <v>46597</v>
+        <v/>
       </c>
       <c r="C23" s="38" t="str">
         <f aca="false">IF(B23="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B23)))</f>
-        <v>חמישי</v>
+        <v/>
       </c>
       <c r="D23" s="40" t="str">
         <f aca="false">IF(B23="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
-        <v>הדרכה 09:00–12:30</v>
+        <v/>
       </c>
       <c r="E23" s="41" t="s">
         <v>83</v>
       </c>
-      <c r="F23" s="42" t="n">
+      <c r="F23" s="42" t="str">
         <f aca="false">IF(B23="","",IF(E23="לא",0,הגדרות!$C$22))</f>
-        <v>3.5</v>
-      </c>
-      <c r="G23" s="43" t="n">
+        <v/>
+      </c>
+      <c r="G23" s="43" t="str">
         <f aca="false">IF(B23="","",F23*הגדרות!$C$24)</f>
-        <v>175</v>
+        <v/>
       </c>
       <c r="H23" s="44"/>
       <c r="I23" s="45"/>
-      <c r="K23" s="27" t="n">
+      <c r="K23" s="27" t="str">
         <f aca="false">IF(B23="","",B23+MIN(MOD(הגדרות!$D$18-WEEKDAY(B23)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B23)-1,7)+1))</f>
-        <v>46600</v>
+        <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4245,7 +4297,7 @@
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="38" t="n">
         <f aca="false">COUNT($B$15:$B$24)+1</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B25" s="46"/>
       <c r="C25" s="38" t="str">
@@ -4280,11 +4332,11 @@
       <c r="E26" s="47"/>
       <c r="F26" s="48" t="n">
         <f aca="false">SUM(F15:F25)</f>
-        <v>32.5</v>
+        <v>29</v>
       </c>
       <c r="G26" s="49" t="n">
         <f aca="false">SUM(G15:G25)</f>
-        <v>1625</v>
+        <v>1450</v>
       </c>
       <c r="H26" s="47"/>
       <c r="I26" s="49" t="n">
@@ -4306,7 +4358,7 @@
       <c r="H28" s="40"/>
       <c r="I28" s="42" t="n">
         <f aca="false">F26</f>
-        <v>32.5</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4320,13 +4372,13 @@
       <c r="E29" s="51"/>
       <c r="F29" s="40" t="str">
         <f aca="false">"הדרכת שיקום ("&amp;TEXT(F26,"0.0")&amp;" שעות × "&amp;הגדרות!$C$24&amp;" ₪)"</f>
-        <v>הדרכת שיקום (32.5 שעות × 50 ₪)</v>
+        <v>הדרכת שיקום (29.0 שעות × 50 ₪)</v>
       </c>
       <c r="G29" s="40"/>
       <c r="H29" s="40"/>
       <c r="I29" s="43" t="n">
         <f aca="false">G26</f>
-        <v>1625</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4364,7 +4416,7 @@
       <c r="H31" s="52"/>
       <c r="I31" s="53" t="n">
         <f aca="false">I29+I30</f>
-        <v>1625</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4384,7 +4436,7 @@
       <c r="H32" s="40"/>
       <c r="I32" s="43" t="n">
         <f aca="false">ROUND(I31*הגדרות!$C$25,2)</f>
-        <v>292.5</v>
+        <v>261</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4395,7 +4447,7 @@
       <c r="H33" s="54"/>
       <c r="I33" s="55" t="n">
         <f aca="false">I31+I32</f>
-        <v>1917.5</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4521,13 +4573,13 @@
       <c r="I1" s="26"/>
       <c r="K1" s="27" t="n">
         <f aca="false">DATE(YEAR($H$11),MONTH($H$11),1)</f>
-        <v>46600</v>
+        <v>46569</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="str">
         <f aca="false">הגדרות!$C$17&amp;" · "&amp;CHOOSE(MONTH($K$1),"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר")&amp;" "&amp;YEAR($K$1)</f>
-        <v>הדרכת שיקום · אוגוסט 2027</v>
+        <v>הדרכת שיקום · יולי 2027</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -4539,7 +4591,7 @@
       <c r="I2" s="28"/>
       <c r="K2" s="27" t="n">
         <f aca="false">EOMONTH($K$1,0)</f>
-        <v>46630</v>
+        <v>46599</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -4647,7 +4699,7 @@
       <c r="B11" s="30"/>
       <c r="C11" s="31" t="str">
         <f aca="false">YEAR($K$1)&amp;"-"&amp;TEXT(MONTH($K$1),"00")</f>
-        <v>2027-08</v>
+        <v>2027-07</v>
       </c>
       <c r="D11" s="31"/>
       <c r="F11" s="30" t="s">
@@ -4655,7 +4707,7 @@
       </c>
       <c r="G11" s="30"/>
       <c r="H11" s="32" t="n">
-        <v>46600</v>
+        <v>46569</v>
       </c>
       <c r="I11" s="32"/>
     </row>
@@ -4666,7 +4718,7 @@
       <c r="B12" s="30"/>
       <c r="C12" s="33" t="n">
         <f aca="false">$K$2</f>
-        <v>46630</v>
+        <v>46599</v>
       </c>
       <c r="D12" s="33"/>
       <c r="F12" s="30" t="s">
@@ -4730,11 +4782,11 @@
       </c>
       <c r="B15" s="39" t="n">
         <f aca="false">$K$1+MIN(MOD(הגדרות!$D$18-WEEKDAY($K$1),7),MOD(הגדרות!$D$19-WEEKDAY($K$1),7))</f>
-        <v>46600</v>
+        <v>46569</v>
       </c>
       <c r="C15" s="38" t="str">
         <f aca="false">IF(B15="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B15)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D15" s="40" t="str">
         <f aca="false">IF(B15="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -4755,7 +4807,7 @@
       <c r="I15" s="45"/>
       <c r="K15" s="27" t="n">
         <f aca="false">IF(B15="","",B15+MIN(MOD(הגדרות!$D$18-WEEKDAY(B15)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B15)-1,7)+1))</f>
-        <v>46604</v>
+        <v>46572</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4765,11 +4817,11 @@
       </c>
       <c r="B16" s="39" t="n">
         <f aca="false">IF(K15="","",IF(K15&gt;$K$2,"",K15))</f>
-        <v>46604</v>
+        <v>46572</v>
       </c>
       <c r="C16" s="38" t="str">
         <f aca="false">IF(B16="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B16)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D16" s="40" t="str">
         <f aca="false">IF(B16="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -4790,7 +4842,7 @@
       <c r="I16" s="45"/>
       <c r="K16" s="27" t="n">
         <f aca="false">IF(B16="","",B16+MIN(MOD(הגדרות!$D$18-WEEKDAY(B16)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B16)-1,7)+1))</f>
-        <v>46607</v>
+        <v>46576</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4800,11 +4852,11 @@
       </c>
       <c r="B17" s="39" t="n">
         <f aca="false">IF(K16="","",IF(K16&gt;$K$2,"",K16))</f>
-        <v>46607</v>
+        <v>46576</v>
       </c>
       <c r="C17" s="38" t="str">
         <f aca="false">IF(B17="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B17)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D17" s="40" t="str">
         <f aca="false">IF(B17="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -4825,7 +4877,7 @@
       <c r="I17" s="45"/>
       <c r="K17" s="27" t="n">
         <f aca="false">IF(B17="","",B17+MIN(MOD(הגדרות!$D$18-WEEKDAY(B17)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B17)-1,7)+1))</f>
-        <v>46611</v>
+        <v>46579</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4835,11 +4887,11 @@
       </c>
       <c r="B18" s="39" t="n">
         <f aca="false">IF(K17="","",IF(K17&gt;$K$2,"",K17))</f>
-        <v>46611</v>
+        <v>46579</v>
       </c>
       <c r="C18" s="38" t="str">
         <f aca="false">IF(B18="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B18)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D18" s="40" t="str">
         <f aca="false">IF(B18="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -4860,7 +4912,7 @@
       <c r="I18" s="45"/>
       <c r="K18" s="27" t="n">
         <f aca="false">IF(B18="","",B18+MIN(MOD(הגדרות!$D$18-WEEKDAY(B18)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B18)-1,7)+1))</f>
-        <v>46614</v>
+        <v>46583</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4870,11 +4922,11 @@
       </c>
       <c r="B19" s="39" t="n">
         <f aca="false">IF(K18="","",IF(K18&gt;$K$2,"",K18))</f>
-        <v>46614</v>
+        <v>46583</v>
       </c>
       <c r="C19" s="38" t="str">
         <f aca="false">IF(B19="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B19)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D19" s="40" t="str">
         <f aca="false">IF(B19="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -4895,7 +4947,7 @@
       <c r="I19" s="45"/>
       <c r="K19" s="27" t="n">
         <f aca="false">IF(B19="","",B19+MIN(MOD(הגדרות!$D$18-WEEKDAY(B19)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B19)-1,7)+1))</f>
-        <v>46618</v>
+        <v>46586</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4905,11 +4957,11 @@
       </c>
       <c r="B20" s="39" t="n">
         <f aca="false">IF(K19="","",IF(K19&gt;$K$2,"",K19))</f>
-        <v>46618</v>
+        <v>46586</v>
       </c>
       <c r="C20" s="38" t="str">
         <f aca="false">IF(B20="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B20)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D20" s="40" t="str">
         <f aca="false">IF(B20="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -4930,7 +4982,7 @@
       <c r="I20" s="45"/>
       <c r="K20" s="27" t="n">
         <f aca="false">IF(B20="","",B20+MIN(MOD(הגדרות!$D$18-WEEKDAY(B20)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B20)-1,7)+1))</f>
-        <v>46621</v>
+        <v>46590</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4940,11 +4992,11 @@
       </c>
       <c r="B21" s="39" t="n">
         <f aca="false">IF(K20="","",IF(K20&gt;$K$2,"",K20))</f>
-        <v>46621</v>
+        <v>46590</v>
       </c>
       <c r="C21" s="38" t="str">
         <f aca="false">IF(B21="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B21)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D21" s="40" t="str">
         <f aca="false">IF(B21="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -4965,7 +5017,7 @@
       <c r="I21" s="45"/>
       <c r="K21" s="27" t="n">
         <f aca="false">IF(B21="","",B21+MIN(MOD(הגדרות!$D$18-WEEKDAY(B21)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B21)-1,7)+1))</f>
-        <v>46625</v>
+        <v>46593</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4975,11 +5027,11 @@
       </c>
       <c r="B22" s="39" t="n">
         <f aca="false">IF(K21="","",IF(K21&gt;$K$2,"",K21))</f>
-        <v>46625</v>
+        <v>46593</v>
       </c>
       <c r="C22" s="38" t="str">
         <f aca="false">IF(B22="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B22)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D22" s="40" t="str">
         <f aca="false">IF(B22="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -5000,7 +5052,7 @@
       <c r="I22" s="45"/>
       <c r="K22" s="27" t="n">
         <f aca="false">IF(B22="","",B22+MIN(MOD(הגדרות!$D$18-WEEKDAY(B22)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B22)-1,7)+1))</f>
-        <v>46628</v>
+        <v>46597</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5010,11 +5062,11 @@
       </c>
       <c r="B23" s="39" t="n">
         <f aca="false">IF(K22="","",IF(K22&gt;$K$2,"",K22))</f>
-        <v>46628</v>
+        <v>46597</v>
       </c>
       <c r="C23" s="38" t="str">
         <f aca="false">IF(B23="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B23)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D23" s="40" t="str">
         <f aca="false">IF(B23="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -5035,7 +5087,7 @@
       <c r="I23" s="45"/>
       <c r="K23" s="27" t="n">
         <f aca="false">IF(B23="","",B23+MIN(MOD(הגדרות!$D$18-WEEKDAY(B23)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B23)-1,7)+1))</f>
-        <v>46632</v>
+        <v>46600</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5352,6 +5404,837 @@
       <c r="I1" s="26"/>
       <c r="K1" s="27" t="n">
         <f aca="false">DATE(YEAR($H$11),MONTH($H$11),1)</f>
+        <v>46600</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="28" t="str">
+        <f aca="false">הגדרות!$C$17&amp;" · "&amp;CHOOSE(MONTH($K$1),"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר")&amp;" "&amp;YEAR($K$1)</f>
+        <v>הדרכת שיקום · אוגוסט 2027</v>
+      </c>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+      <c r="K2" s="27" t="n">
+        <f aca="false">EOMONTH($K$1,0)</f>
+        <v>46630</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="29" t="s">
+        <v>68</v>
+      </c>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="F4" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="G4" s="29"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="29"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="30"/>
+      <c r="C5" s="31" t="str">
+        <f aca="false">הגדרות!$C$5</f>
+        <v>הנגרייה</v>
+      </c>
+      <c r="D5" s="31"/>
+      <c r="F5" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" s="30"/>
+      <c r="H5" s="31" t="str">
+        <f aca="false">הגדרות!$C$12</f>
+        <v>חוות רום</v>
+      </c>
+      <c r="I5" s="31"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="30"/>
+      <c r="C6" s="31" t="str">
+        <f aca="false">הגדרות!$C$6</f>
+        <v>(למילוי)</v>
+      </c>
+      <c r="D6" s="31"/>
+      <c r="F6" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="30"/>
+      <c r="H6" s="31" t="str">
+        <f aca="false">הגדרות!$C$13</f>
+        <v>הר כמון</v>
+      </c>
+      <c r="I6" s="31"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="30"/>
+      <c r="C7" s="31" t="str">
+        <f aca="false">הגדרות!$C$7</f>
+        <v>(למילוי)</v>
+      </c>
+      <c r="D7" s="31"/>
+      <c r="F7" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="30"/>
+      <c r="H7" s="31" t="str">
+        <f aca="false">הגדרות!$C$14</f>
+        <v>(למילוי)</v>
+      </c>
+      <c r="I7" s="31"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="30"/>
+      <c r="C8" s="31" t="str">
+        <f aca="false">הגדרות!$C$8</f>
+        <v>(למילוי)</v>
+      </c>
+      <c r="D8" s="31"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="30"/>
+      <c r="C9" s="31" t="str">
+        <f aca="false">הגדרות!$C$9</f>
+        <v>nettaamit21@gmail.com</v>
+      </c>
+      <c r="D9" s="31"/>
+    </row>
+    <row r="10" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="30"/>
+      <c r="C11" s="31" t="str">
+        <f aca="false">YEAR($K$1)&amp;"-"&amp;TEXT(MONTH($K$1),"00")</f>
+        <v>2027-08</v>
+      </c>
+      <c r="D11" s="31"/>
+      <c r="F11" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="G11" s="30"/>
+      <c r="H11" s="32" t="n">
+        <v>46600</v>
+      </c>
+      <c r="I11" s="32"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="30"/>
+      <c r="C12" s="33" t="n">
+        <f aca="false">$K$2</f>
+        <v>46630</v>
+      </c>
+      <c r="D12" s="33"/>
+      <c r="F12" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="G12" s="30"/>
+      <c r="H12" s="31" t="str">
+        <f aca="false">הגדרות!$C$18&amp;" ו"&amp;הגדרות!$C$19&amp;", "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00")</f>
+        <v>ראשון וחמישי, 09:00–12:30</v>
+      </c>
+      <c r="I12" s="31"/>
+    </row>
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" s="34"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="35" t="s">
+        <v>76</v>
+      </c>
+      <c r="I13" s="35"/>
+    </row>
+    <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="36" t="s">
+        <v>77</v>
+      </c>
+      <c r="B14" s="36" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="E14" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="F14" s="36" t="s">
+        <v>81</v>
+      </c>
+      <c r="G14" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="H14" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="I14" s="37" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="38" t="n">
+        <f aca="false">IF(B15="","",ROW()-14)</f>
+        <v>1</v>
+      </c>
+      <c r="B15" s="39" t="n">
+        <f aca="false">$K$1+MIN(MOD(הגדרות!$D$18-WEEKDAY($K$1),7),MOD(הגדרות!$D$19-WEEKDAY($K$1),7))</f>
+        <v>46600</v>
+      </c>
+      <c r="C15" s="38" t="str">
+        <f aca="false">IF(B15="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B15)))</f>
+        <v>ראשון</v>
+      </c>
+      <c r="D15" s="40" t="str">
+        <f aca="false">IF(B15="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
+        <v>הדרכה 09:00–12:30</v>
+      </c>
+      <c r="E15" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="F15" s="42" t="n">
+        <f aca="false">IF(B15="","",IF(E15="לא",0,הגדרות!$C$22))</f>
+        <v>3.5</v>
+      </c>
+      <c r="G15" s="43" t="n">
+        <f aca="false">IF(B15="","",F15*הגדרות!$C$24)</f>
+        <v>175</v>
+      </c>
+      <c r="H15" s="44"/>
+      <c r="I15" s="45"/>
+      <c r="K15" s="27" t="n">
+        <f aca="false">IF(B15="","",B15+MIN(MOD(הגדרות!$D$18-WEEKDAY(B15)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B15)-1,7)+1))</f>
+        <v>46604</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="38" t="n">
+        <f aca="false">IF(B16="","",ROW()-14)</f>
+        <v>2</v>
+      </c>
+      <c r="B16" s="39" t="n">
+        <f aca="false">IF(K15="","",IF(K15&gt;$K$2,"",K15))</f>
+        <v>46604</v>
+      </c>
+      <c r="C16" s="38" t="str">
+        <f aca="false">IF(B16="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B16)))</f>
+        <v>חמישי</v>
+      </c>
+      <c r="D16" s="40" t="str">
+        <f aca="false">IF(B16="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
+        <v>הדרכה 09:00–12:30</v>
+      </c>
+      <c r="E16" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" s="42" t="n">
+        <f aca="false">IF(B16="","",IF(E16="לא",0,הגדרות!$C$22))</f>
+        <v>3.5</v>
+      </c>
+      <c r="G16" s="43" t="n">
+        <f aca="false">IF(B16="","",F16*הגדרות!$C$24)</f>
+        <v>175</v>
+      </c>
+      <c r="H16" s="44"/>
+      <c r="I16" s="45"/>
+      <c r="K16" s="27" t="n">
+        <f aca="false">IF(B16="","",B16+MIN(MOD(הגדרות!$D$18-WEEKDAY(B16)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B16)-1,7)+1))</f>
+        <v>46607</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="38" t="n">
+        <f aca="false">IF(B17="","",ROW()-14)</f>
+        <v>3</v>
+      </c>
+      <c r="B17" s="39" t="n">
+        <f aca="false">IF(K16="","",IF(K16&gt;$K$2,"",K16))</f>
+        <v>46607</v>
+      </c>
+      <c r="C17" s="38" t="str">
+        <f aca="false">IF(B17="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B17)))</f>
+        <v>ראשון</v>
+      </c>
+      <c r="D17" s="40" t="str">
+        <f aca="false">IF(B17="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
+        <v>הדרכה 09:00–12:30</v>
+      </c>
+      <c r="E17" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="F17" s="42" t="n">
+        <f aca="false">IF(B17="","",IF(E17="לא",0,הגדרות!$C$22))</f>
+        <v>3.5</v>
+      </c>
+      <c r="G17" s="43" t="n">
+        <f aca="false">IF(B17="","",F17*הגדרות!$C$24)</f>
+        <v>175</v>
+      </c>
+      <c r="H17" s="44"/>
+      <c r="I17" s="45"/>
+      <c r="K17" s="27" t="n">
+        <f aca="false">IF(B17="","",B17+MIN(MOD(הגדרות!$D$18-WEEKDAY(B17)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B17)-1,7)+1))</f>
+        <v>46611</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="38" t="n">
+        <f aca="false">IF(B18="","",ROW()-14)</f>
+        <v>4</v>
+      </c>
+      <c r="B18" s="39" t="n">
+        <f aca="false">IF(K17="","",IF(K17&gt;$K$2,"",K17))</f>
+        <v>46611</v>
+      </c>
+      <c r="C18" s="38" t="str">
+        <f aca="false">IF(B18="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B18)))</f>
+        <v>חמישי</v>
+      </c>
+      <c r="D18" s="40" t="str">
+        <f aca="false">IF(B18="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
+        <v>הדרכה 09:00–12:30</v>
+      </c>
+      <c r="E18" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="F18" s="42" t="n">
+        <f aca="false">IF(B18="","",IF(E18="לא",0,הגדרות!$C$22))</f>
+        <v>3.5</v>
+      </c>
+      <c r="G18" s="43" t="n">
+        <f aca="false">IF(B18="","",F18*הגדרות!$C$24)</f>
+        <v>175</v>
+      </c>
+      <c r="H18" s="44"/>
+      <c r="I18" s="45"/>
+      <c r="K18" s="27" t="n">
+        <f aca="false">IF(B18="","",B18+MIN(MOD(הגדרות!$D$18-WEEKDAY(B18)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B18)-1,7)+1))</f>
+        <v>46614</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="38" t="n">
+        <f aca="false">IF(B19="","",ROW()-14)</f>
+        <v>5</v>
+      </c>
+      <c r="B19" s="39" t="n">
+        <f aca="false">IF(K18="","",IF(K18&gt;$K$2,"",K18))</f>
+        <v>46614</v>
+      </c>
+      <c r="C19" s="38" t="str">
+        <f aca="false">IF(B19="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B19)))</f>
+        <v>ראשון</v>
+      </c>
+      <c r="D19" s="40" t="str">
+        <f aca="false">IF(B19="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
+        <v>הדרכה 09:00–12:30</v>
+      </c>
+      <c r="E19" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="F19" s="42" t="n">
+        <f aca="false">IF(B19="","",IF(E19="לא",0,הגדרות!$C$22))</f>
+        <v>3.5</v>
+      </c>
+      <c r="G19" s="43" t="n">
+        <f aca="false">IF(B19="","",F19*הגדרות!$C$24)</f>
+        <v>175</v>
+      </c>
+      <c r="H19" s="44"/>
+      <c r="I19" s="45"/>
+      <c r="K19" s="27" t="n">
+        <f aca="false">IF(B19="","",B19+MIN(MOD(הגדרות!$D$18-WEEKDAY(B19)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B19)-1,7)+1))</f>
+        <v>46618</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="38" t="n">
+        <f aca="false">IF(B20="","",ROW()-14)</f>
+        <v>6</v>
+      </c>
+      <c r="B20" s="39" t="n">
+        <f aca="false">IF(K19="","",IF(K19&gt;$K$2,"",K19))</f>
+        <v>46618</v>
+      </c>
+      <c r="C20" s="38" t="str">
+        <f aca="false">IF(B20="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B20)))</f>
+        <v>חמישי</v>
+      </c>
+      <c r="D20" s="40" t="str">
+        <f aca="false">IF(B20="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
+        <v>הדרכה 09:00–12:30</v>
+      </c>
+      <c r="E20" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="F20" s="42" t="n">
+        <f aca="false">IF(B20="","",IF(E20="לא",0,הגדרות!$C$22))</f>
+        <v>3.5</v>
+      </c>
+      <c r="G20" s="43" t="n">
+        <f aca="false">IF(B20="","",F20*הגדרות!$C$24)</f>
+        <v>175</v>
+      </c>
+      <c r="H20" s="44"/>
+      <c r="I20" s="45"/>
+      <c r="K20" s="27" t="n">
+        <f aca="false">IF(B20="","",B20+MIN(MOD(הגדרות!$D$18-WEEKDAY(B20)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B20)-1,7)+1))</f>
+        <v>46621</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="38" t="n">
+        <f aca="false">IF(B21="","",ROW()-14)</f>
+        <v>7</v>
+      </c>
+      <c r="B21" s="39" t="n">
+        <f aca="false">IF(K20="","",IF(K20&gt;$K$2,"",K20))</f>
+        <v>46621</v>
+      </c>
+      <c r="C21" s="38" t="str">
+        <f aca="false">IF(B21="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B21)))</f>
+        <v>ראשון</v>
+      </c>
+      <c r="D21" s="40" t="str">
+        <f aca="false">IF(B21="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
+        <v>הדרכה 09:00–12:30</v>
+      </c>
+      <c r="E21" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="F21" s="42" t="n">
+        <f aca="false">IF(B21="","",IF(E21="לא",0,הגדרות!$C$22))</f>
+        <v>3.5</v>
+      </c>
+      <c r="G21" s="43" t="n">
+        <f aca="false">IF(B21="","",F21*הגדרות!$C$24)</f>
+        <v>175</v>
+      </c>
+      <c r="H21" s="44"/>
+      <c r="I21" s="45"/>
+      <c r="K21" s="27" t="n">
+        <f aca="false">IF(B21="","",B21+MIN(MOD(הגדרות!$D$18-WEEKDAY(B21)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B21)-1,7)+1))</f>
+        <v>46625</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="38" t="n">
+        <f aca="false">IF(B22="","",ROW()-14)</f>
+        <v>8</v>
+      </c>
+      <c r="B22" s="39" t="n">
+        <f aca="false">IF(K21="","",IF(K21&gt;$K$2,"",K21))</f>
+        <v>46625</v>
+      </c>
+      <c r="C22" s="38" t="str">
+        <f aca="false">IF(B22="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B22)))</f>
+        <v>חמישי</v>
+      </c>
+      <c r="D22" s="40" t="str">
+        <f aca="false">IF(B22="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
+        <v>הדרכה 09:00–12:30</v>
+      </c>
+      <c r="E22" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="F22" s="42" t="n">
+        <f aca="false">IF(B22="","",IF(E22="לא",0,הגדרות!$C$22))</f>
+        <v>3.5</v>
+      </c>
+      <c r="G22" s="43" t="n">
+        <f aca="false">IF(B22="","",F22*הגדרות!$C$24)</f>
+        <v>175</v>
+      </c>
+      <c r="H22" s="44"/>
+      <c r="I22" s="45"/>
+      <c r="K22" s="27" t="n">
+        <f aca="false">IF(B22="","",B22+MIN(MOD(הגדרות!$D$18-WEEKDAY(B22)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B22)-1,7)+1))</f>
+        <v>46628</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="38" t="n">
+        <f aca="false">IF(B23="","",ROW()-14)</f>
+        <v>9</v>
+      </c>
+      <c r="B23" s="39" t="n">
+        <f aca="false">IF(K22="","",IF(K22&gt;$K$2,"",K22))</f>
+        <v>46628</v>
+      </c>
+      <c r="C23" s="38" t="str">
+        <f aca="false">IF(B23="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B23)))</f>
+        <v>ראשון</v>
+      </c>
+      <c r="D23" s="40" t="str">
+        <f aca="false">IF(B23="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
+        <v>הדרכה 09:00–12:30</v>
+      </c>
+      <c r="E23" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="F23" s="42" t="n">
+        <f aca="false">IF(B23="","",IF(E23="לא",0,הגדרות!$C$22))</f>
+        <v>3.5</v>
+      </c>
+      <c r="G23" s="43" t="n">
+        <f aca="false">IF(B23="","",F23*הגדרות!$C$24)</f>
+        <v>175</v>
+      </c>
+      <c r="H23" s="44"/>
+      <c r="I23" s="45"/>
+      <c r="K23" s="27" t="n">
+        <f aca="false">IF(B23="","",B23+MIN(MOD(הגדרות!$D$18-WEEKDAY(B23)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B23)-1,7)+1))</f>
+        <v>46632</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="38" t="str">
+        <f aca="false">IF(B24="","",ROW()-14)</f>
+        <v/>
+      </c>
+      <c r="B24" s="39" t="str">
+        <f aca="false">IF(K23="","",IF(K23&gt;$K$2,"",K23))</f>
+        <v/>
+      </c>
+      <c r="C24" s="38" t="str">
+        <f aca="false">IF(B24="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B24)))</f>
+        <v/>
+      </c>
+      <c r="D24" s="40" t="str">
+        <f aca="false">IF(B24="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
+        <v/>
+      </c>
+      <c r="E24" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="F24" s="42" t="str">
+        <f aca="false">IF(B24="","",IF(E24="לא",0,הגדרות!$C$22))</f>
+        <v/>
+      </c>
+      <c r="G24" s="43" t="str">
+        <f aca="false">IF(B24="","",F24*הגדרות!$C$24)</f>
+        <v/>
+      </c>
+      <c r="H24" s="44"/>
+      <c r="I24" s="45"/>
+      <c r="K24" s="27" t="str">
+        <f aca="false">IF(B24="","",B24+MIN(MOD(הגדרות!$D$18-WEEKDAY(B24)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B24)-1,7)+1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="38" t="n">
+        <f aca="false">COUNT($B$15:$B$24)+1</f>
+        <v>10</v>
+      </c>
+      <c r="B25" s="46"/>
+      <c r="C25" s="38" t="str">
+        <f aca="false">IF(B25="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B25)))</f>
+        <v/>
+      </c>
+      <c r="D25" s="40" t="s">
+        <v>84</v>
+      </c>
+      <c r="E25" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="F25" s="42" t="n">
+        <f aca="false">IF(E25="לא",0,הגדרות!$C$23)</f>
+        <v>1</v>
+      </c>
+      <c r="G25" s="43" t="n">
+        <f aca="false">F25*הגדרות!$C$24</f>
+        <v>50</v>
+      </c>
+      <c r="H25" s="44"/>
+      <c r="I25" s="45"/>
+      <c r="K25" s="27"/>
+    </row>
+    <row r="26" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="47" t="s">
+        <v>85</v>
+      </c>
+      <c r="B26" s="47"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="47"/>
+      <c r="E26" s="47"/>
+      <c r="F26" s="48" t="n">
+        <f aca="false">SUM(F15:F25)</f>
+        <v>32.5</v>
+      </c>
+      <c r="G26" s="49" t="n">
+        <f aca="false">SUM(G15:G25)</f>
+        <v>1625</v>
+      </c>
+      <c r="H26" s="47"/>
+      <c r="I26" s="49" t="n">
+        <f aca="false">SUM(I15:I25)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="50" t="s">
+        <v>86</v>
+      </c>
+      <c r="B28" s="50"/>
+      <c r="C28" s="50"/>
+      <c r="D28" s="50"/>
+      <c r="F28" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G28" s="40"/>
+      <c r="H28" s="40"/>
+      <c r="I28" s="42" t="n">
+        <f aca="false">F26</f>
+        <v>32.5</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="51" t="str">
+        <f aca="false">"• "&amp;הגדרות!$C$17&amp;": ימי "&amp;הגדרות!$C$18&amp;" ו"&amp;הגדרות!$C$19&amp;", "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00")&amp;" ("&amp;הגדרות!$C$22&amp;" שעות ליום), וישיבת צוות חודשית ("&amp;הגדרות!$C$23&amp;" ש׳)."</f>
+        <v>• הדרכת שיקום: ימי ראשון וחמישי, 09:00–12:30 (3.5 שעות ליום), וישיבת צוות חודשית (1 ש׳).</v>
+      </c>
+      <c r="B29" s="51"/>
+      <c r="C29" s="51"/>
+      <c r="D29" s="51"/>
+      <c r="E29" s="51"/>
+      <c r="F29" s="40" t="str">
+        <f aca="false">"הדרכת שיקום ("&amp;TEXT(F26,"0.0")&amp;" שעות × "&amp;הגדרות!$C$24&amp;" ₪)"</f>
+        <v>הדרכת שיקום (32.5 שעות × 50 ₪)</v>
+      </c>
+      <c r="G29" s="40"/>
+      <c r="H29" s="40"/>
+      <c r="I29" s="43" t="n">
+        <f aca="false">G26</f>
+        <v>1625</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="51" t="str">
+        <f aca="false">IF(הגדרות!$C$28="","","• "&amp;הגדרות!$C$28)</f>
+        <v>• התעריף השעתי אינו כולל מע״מ. מע״מ יתווסף כחוק.</v>
+      </c>
+      <c r="B30" s="51"/>
+      <c r="C30" s="51"/>
+      <c r="D30" s="51"/>
+      <c r="E30" s="51"/>
+      <c r="F30" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="G30" s="40"/>
+      <c r="H30" s="40"/>
+      <c r="I30" s="43" t="n">
+        <f aca="false">I26</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="51" t="str">
+        <f aca="false">IF(הגדרות!$C$29="","","• "&amp;הגדרות!$C$29)</f>
+        <v>• פרויקטים פרטיים מתומחרים בנפרד, לפי הזמנת החווה.</v>
+      </c>
+      <c r="B31" s="51"/>
+      <c r="C31" s="51"/>
+      <c r="D31" s="51"/>
+      <c r="E31" s="51"/>
+      <c r="F31" s="52" t="s">
+        <v>89</v>
+      </c>
+      <c r="G31" s="52"/>
+      <c r="H31" s="52"/>
+      <c r="I31" s="53" t="n">
+        <f aca="false">I29+I30</f>
+        <v>1625</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="51" t="str">
+        <f aca="false">IF(הגדרות!$C$30="","","• "&amp;הגדרות!$C$30)</f>
+        <v/>
+      </c>
+      <c r="B32" s="51"/>
+      <c r="C32" s="51"/>
+      <c r="D32" s="51"/>
+      <c r="E32" s="51"/>
+      <c r="F32" s="40" t="str">
+        <f aca="false">"מע״מ "&amp;ROUND(הגדרות!$C$25*100,1)&amp;"%"</f>
+        <v>מע״מ 18%</v>
+      </c>
+      <c r="G32" s="40"/>
+      <c r="H32" s="40"/>
+      <c r="I32" s="43" t="n">
+        <f aca="false">ROUND(I31*הגדרות!$C$25,2)</f>
+        <v>292.5</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F33" s="54" t="s">
+        <v>90</v>
+      </c>
+      <c r="G33" s="54"/>
+      <c r="H33" s="54"/>
+      <c r="I33" s="55" t="n">
+        <f aca="false">I31+I32</f>
+        <v>1917.5</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="56" t="str">
+        <f aca="false">"בברכה, "&amp;הגדרות!$C$6</f>
+        <v>בברכה, (למילוי)</v>
+      </c>
+      <c r="B36" s="56"/>
+      <c r="C36" s="56"/>
+      <c r="D36" s="56"/>
+      <c r="F36" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="G36" s="56"/>
+      <c r="H36" s="56"/>
+      <c r="I36" s="56"/>
+    </row>
+  </sheetData>
+  <mergeCells count="44">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="F28:H28"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="F29:H29"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="F31:H31"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="F33:H33"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="F36:I36"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E15:E24">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>$B15=""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A15:G25">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>$E15="לא"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E15:E25" type="list">
+      <formula1>"כן,לא"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:K36"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="11" min="11" style="0" width="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="K1" s="27" t="n">
+        <f aca="false">DATE(YEAR($H$11),MONTH($H$11),1)</f>
         <v>46631</v>
       </c>
     </row>
@@ -6447,13 +7330,13 @@
       <c r="I1" s="26"/>
       <c r="K1" s="27" t="n">
         <f aca="false">DATE(YEAR($H$11),MONTH($H$11),1)</f>
-        <v>46296</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="str">
         <f aca="false">הגדרות!$C$17&amp;" · "&amp;CHOOSE(MONTH($K$1),"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר")&amp;" "&amp;YEAR($K$1)</f>
-        <v>הדרכת שיקום · אוקטובר 2026</v>
+        <v>הדרכת שיקום · ספטמבר 2026</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -6465,7 +7348,7 @@
       <c r="I2" s="28"/>
       <c r="K2" s="27" t="n">
         <f aca="false">EOMONTH($K$1,0)</f>
-        <v>46326</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -6573,7 +7456,7 @@
       <c r="B11" s="30"/>
       <c r="C11" s="31" t="str">
         <f aca="false">YEAR($K$1)&amp;"-"&amp;TEXT(MONTH($K$1),"00")</f>
-        <v>2026-10</v>
+        <v>2026-09</v>
       </c>
       <c r="D11" s="31"/>
       <c r="F11" s="30" t="s">
@@ -6581,7 +7464,7 @@
       </c>
       <c r="G11" s="30"/>
       <c r="H11" s="32" t="n">
-        <v>46296</v>
+        <v>46266</v>
       </c>
       <c r="I11" s="32"/>
     </row>
@@ -6592,7 +7475,7 @@
       <c r="B12" s="30"/>
       <c r="C12" s="33" t="n">
         <f aca="false">$K$2</f>
-        <v>46326</v>
+        <v>46295</v>
       </c>
       <c r="D12" s="33"/>
       <c r="F12" s="30" t="s">
@@ -6656,7 +7539,7 @@
       </c>
       <c r="B15" s="39" t="n">
         <f aca="false">$K$1+MIN(MOD(הגדרות!$D$18-WEEKDAY($K$1),7),MOD(הגדרות!$D$19-WEEKDAY($K$1),7))</f>
-        <v>46296</v>
+        <v>46268</v>
       </c>
       <c r="C15" s="38" t="str">
         <f aca="false">IF(B15="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B15)))</f>
@@ -6681,7 +7564,7 @@
       <c r="I15" s="45"/>
       <c r="K15" s="27" t="n">
         <f aca="false">IF(B15="","",B15+MIN(MOD(הגדרות!$D$18-WEEKDAY(B15)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B15)-1,7)+1))</f>
-        <v>46299</v>
+        <v>46271</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6691,7 +7574,7 @@
       </c>
       <c r="B16" s="39" t="n">
         <f aca="false">IF(K15="","",IF(K15&gt;$K$2,"",K15))</f>
-        <v>46299</v>
+        <v>46271</v>
       </c>
       <c r="C16" s="38" t="str">
         <f aca="false">IF(B16="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B16)))</f>
@@ -6716,7 +7599,7 @@
       <c r="I16" s="45"/>
       <c r="K16" s="27" t="n">
         <f aca="false">IF(B16="","",B16+MIN(MOD(הגדרות!$D$18-WEEKDAY(B16)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B16)-1,7)+1))</f>
-        <v>46303</v>
+        <v>46275</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6726,7 +7609,7 @@
       </c>
       <c r="B17" s="39" t="n">
         <f aca="false">IF(K16="","",IF(K16&gt;$K$2,"",K16))</f>
-        <v>46303</v>
+        <v>46275</v>
       </c>
       <c r="C17" s="38" t="str">
         <f aca="false">IF(B17="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B17)))</f>
@@ -6751,7 +7634,7 @@
       <c r="I17" s="45"/>
       <c r="K17" s="27" t="n">
         <f aca="false">IF(B17="","",B17+MIN(MOD(הגדרות!$D$18-WEEKDAY(B17)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B17)-1,7)+1))</f>
-        <v>46306</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6761,7 +7644,7 @@
       </c>
       <c r="B18" s="39" t="n">
         <f aca="false">IF(K17="","",IF(K17&gt;$K$2,"",K17))</f>
-        <v>46306</v>
+        <v>46278</v>
       </c>
       <c r="C18" s="38" t="str">
         <f aca="false">IF(B18="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B18)))</f>
@@ -6786,7 +7669,7 @@
       <c r="I18" s="45"/>
       <c r="K18" s="27" t="n">
         <f aca="false">IF(B18="","",B18+MIN(MOD(הגדרות!$D$18-WEEKDAY(B18)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B18)-1,7)+1))</f>
-        <v>46310</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6796,7 +7679,7 @@
       </c>
       <c r="B19" s="39" t="n">
         <f aca="false">IF(K18="","",IF(K18&gt;$K$2,"",K18))</f>
-        <v>46310</v>
+        <v>46282</v>
       </c>
       <c r="C19" s="38" t="str">
         <f aca="false">IF(B19="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B19)))</f>
@@ -6821,7 +7704,7 @@
       <c r="I19" s="45"/>
       <c r="K19" s="27" t="n">
         <f aca="false">IF(B19="","",B19+MIN(MOD(הגדרות!$D$18-WEEKDAY(B19)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B19)-1,7)+1))</f>
-        <v>46313</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6831,7 +7714,7 @@
       </c>
       <c r="B20" s="39" t="n">
         <f aca="false">IF(K19="","",IF(K19&gt;$K$2,"",K19))</f>
-        <v>46313</v>
+        <v>46285</v>
       </c>
       <c r="C20" s="38" t="str">
         <f aca="false">IF(B20="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B20)))</f>
@@ -6856,7 +7739,7 @@
       <c r="I20" s="45"/>
       <c r="K20" s="27" t="n">
         <f aca="false">IF(B20="","",B20+MIN(MOD(הגדרות!$D$18-WEEKDAY(B20)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B20)-1,7)+1))</f>
-        <v>46317</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6866,7 +7749,7 @@
       </c>
       <c r="B21" s="39" t="n">
         <f aca="false">IF(K20="","",IF(K20&gt;$K$2,"",K20))</f>
-        <v>46317</v>
+        <v>46289</v>
       </c>
       <c r="C21" s="38" t="str">
         <f aca="false">IF(B21="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B21)))</f>
@@ -6891,7 +7774,7 @@
       <c r="I21" s="45"/>
       <c r="K21" s="27" t="n">
         <f aca="false">IF(B21="","",B21+MIN(MOD(הגדרות!$D$18-WEEKDAY(B21)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B21)-1,7)+1))</f>
-        <v>46320</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6901,7 +7784,7 @@
       </c>
       <c r="B22" s="39" t="n">
         <f aca="false">IF(K21="","",IF(K21&gt;$K$2,"",K21))</f>
-        <v>46320</v>
+        <v>46292</v>
       </c>
       <c r="C22" s="38" t="str">
         <f aca="false">IF(B22="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B22)))</f>
@@ -6926,42 +7809,42 @@
       <c r="I22" s="45"/>
       <c r="K22" s="27" t="n">
         <f aca="false">IF(B22="","",B22+MIN(MOD(הגדרות!$D$18-WEEKDAY(B22)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B22)-1,7)+1))</f>
-        <v>46324</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="38" t="n">
+      <c r="A23" s="38" t="str">
         <f aca="false">IF(B23="","",ROW()-14)</f>
-        <v>9</v>
-      </c>
-      <c r="B23" s="39" t="n">
+        <v/>
+      </c>
+      <c r="B23" s="39" t="str">
         <f aca="false">IF(K22="","",IF(K22&gt;$K$2,"",K22))</f>
-        <v>46324</v>
+        <v/>
       </c>
       <c r="C23" s="38" t="str">
         <f aca="false">IF(B23="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B23)))</f>
-        <v>חמישי</v>
+        <v/>
       </c>
       <c r="D23" s="40" t="str">
         <f aca="false">IF(B23="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
-        <v>הדרכה 09:00–12:30</v>
+        <v/>
       </c>
       <c r="E23" s="41" t="s">
         <v>83</v>
       </c>
-      <c r="F23" s="42" t="n">
+      <c r="F23" s="42" t="str">
         <f aca="false">IF(B23="","",IF(E23="לא",0,הגדרות!$C$22))</f>
-        <v>3.5</v>
-      </c>
-      <c r="G23" s="43" t="n">
+        <v/>
+      </c>
+      <c r="G23" s="43" t="str">
         <f aca="false">IF(B23="","",F23*הגדרות!$C$24)</f>
-        <v>175</v>
+        <v/>
       </c>
       <c r="H23" s="44"/>
       <c r="I23" s="45"/>
-      <c r="K23" s="27" t="n">
+      <c r="K23" s="27" t="str">
         <f aca="false">IF(B23="","",B23+MIN(MOD(הגדרות!$D$18-WEEKDAY(B23)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B23)-1,7)+1))</f>
-        <v>46327</v>
+        <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7002,7 +7885,7 @@
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="38" t="n">
         <f aca="false">COUNT($B$15:$B$24)+1</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B25" s="46"/>
       <c r="C25" s="38" t="str">
@@ -7037,11 +7920,11 @@
       <c r="E26" s="47"/>
       <c r="F26" s="48" t="n">
         <f aca="false">SUM(F15:F25)</f>
-        <v>32.5</v>
+        <v>29</v>
       </c>
       <c r="G26" s="49" t="n">
         <f aca="false">SUM(G15:G25)</f>
-        <v>1625</v>
+        <v>1450</v>
       </c>
       <c r="H26" s="47"/>
       <c r="I26" s="49" t="n">
@@ -7063,7 +7946,7 @@
       <c r="H28" s="40"/>
       <c r="I28" s="42" t="n">
         <f aca="false">F26</f>
-        <v>32.5</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7077,13 +7960,13 @@
       <c r="E29" s="51"/>
       <c r="F29" s="40" t="str">
         <f aca="false">"הדרכת שיקום ("&amp;TEXT(F26,"0.0")&amp;" שעות × "&amp;הגדרות!$C$24&amp;" ₪)"</f>
-        <v>הדרכת שיקום (32.5 שעות × 50 ₪)</v>
+        <v>הדרכת שיקום (29.0 שעות × 50 ₪)</v>
       </c>
       <c r="G29" s="40"/>
       <c r="H29" s="40"/>
       <c r="I29" s="43" t="n">
         <f aca="false">G26</f>
-        <v>1625</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7121,7 +8004,7 @@
       <c r="H31" s="52"/>
       <c r="I31" s="53" t="n">
         <f aca="false">I29+I30</f>
-        <v>1625</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7141,7 +8024,7 @@
       <c r="H32" s="40"/>
       <c r="I32" s="43" t="n">
         <f aca="false">ROUND(I31*הגדרות!$C$25,2)</f>
-        <v>292.5</v>
+        <v>261</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7152,7 +8035,7 @@
       <c r="H33" s="54"/>
       <c r="I33" s="55" t="n">
         <f aca="false">I31+I32</f>
-        <v>1917.5</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7278,13 +8161,13 @@
       <c r="I1" s="26"/>
       <c r="K1" s="27" t="n">
         <f aca="false">DATE(YEAR($H$11),MONTH($H$11),1)</f>
-        <v>46327</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="str">
         <f aca="false">הגדרות!$C$17&amp;" · "&amp;CHOOSE(MONTH($K$1),"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר")&amp;" "&amp;YEAR($K$1)</f>
-        <v>הדרכת שיקום · נובמבר 2026</v>
+        <v>הדרכת שיקום · אוקטובר 2026</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -7296,7 +8179,7 @@
       <c r="I2" s="28"/>
       <c r="K2" s="27" t="n">
         <f aca="false">EOMONTH($K$1,0)</f>
-        <v>46356</v>
+        <v>46326</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -7404,7 +8287,7 @@
       <c r="B11" s="30"/>
       <c r="C11" s="31" t="str">
         <f aca="false">YEAR($K$1)&amp;"-"&amp;TEXT(MONTH($K$1),"00")</f>
-        <v>2026-11</v>
+        <v>2026-10</v>
       </c>
       <c r="D11" s="31"/>
       <c r="F11" s="30" t="s">
@@ -7412,7 +8295,7 @@
       </c>
       <c r="G11" s="30"/>
       <c r="H11" s="32" t="n">
-        <v>46327</v>
+        <v>46296</v>
       </c>
       <c r="I11" s="32"/>
     </row>
@@ -7423,7 +8306,7 @@
       <c r="B12" s="30"/>
       <c r="C12" s="33" t="n">
         <f aca="false">$K$2</f>
-        <v>46356</v>
+        <v>46326</v>
       </c>
       <c r="D12" s="33"/>
       <c r="F12" s="30" t="s">
@@ -7487,11 +8370,11 @@
       </c>
       <c r="B15" s="39" t="n">
         <f aca="false">$K$1+MIN(MOD(הגדרות!$D$18-WEEKDAY($K$1),7),MOD(הגדרות!$D$19-WEEKDAY($K$1),7))</f>
-        <v>46327</v>
+        <v>46296</v>
       </c>
       <c r="C15" s="38" t="str">
         <f aca="false">IF(B15="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B15)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D15" s="40" t="str">
         <f aca="false">IF(B15="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -7512,7 +8395,7 @@
       <c r="I15" s="45"/>
       <c r="K15" s="27" t="n">
         <f aca="false">IF(B15="","",B15+MIN(MOD(הגדרות!$D$18-WEEKDAY(B15)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B15)-1,7)+1))</f>
-        <v>46331</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7522,11 +8405,11 @@
       </c>
       <c r="B16" s="39" t="n">
         <f aca="false">IF(K15="","",IF(K15&gt;$K$2,"",K15))</f>
-        <v>46331</v>
+        <v>46299</v>
       </c>
       <c r="C16" s="38" t="str">
         <f aca="false">IF(B16="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B16)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D16" s="40" t="str">
         <f aca="false">IF(B16="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -7547,7 +8430,7 @@
       <c r="I16" s="45"/>
       <c r="K16" s="27" t="n">
         <f aca="false">IF(B16="","",B16+MIN(MOD(הגדרות!$D$18-WEEKDAY(B16)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B16)-1,7)+1))</f>
-        <v>46334</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7557,11 +8440,11 @@
       </c>
       <c r="B17" s="39" t="n">
         <f aca="false">IF(K16="","",IF(K16&gt;$K$2,"",K16))</f>
-        <v>46334</v>
+        <v>46303</v>
       </c>
       <c r="C17" s="38" t="str">
         <f aca="false">IF(B17="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B17)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D17" s="40" t="str">
         <f aca="false">IF(B17="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -7582,7 +8465,7 @@
       <c r="I17" s="45"/>
       <c r="K17" s="27" t="n">
         <f aca="false">IF(B17="","",B17+MIN(MOD(הגדרות!$D$18-WEEKDAY(B17)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B17)-1,7)+1))</f>
-        <v>46338</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7592,11 +8475,11 @@
       </c>
       <c r="B18" s="39" t="n">
         <f aca="false">IF(K17="","",IF(K17&gt;$K$2,"",K17))</f>
-        <v>46338</v>
+        <v>46306</v>
       </c>
       <c r="C18" s="38" t="str">
         <f aca="false">IF(B18="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B18)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D18" s="40" t="str">
         <f aca="false">IF(B18="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -7617,7 +8500,7 @@
       <c r="I18" s="45"/>
       <c r="K18" s="27" t="n">
         <f aca="false">IF(B18="","",B18+MIN(MOD(הגדרות!$D$18-WEEKDAY(B18)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B18)-1,7)+1))</f>
-        <v>46341</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7627,11 +8510,11 @@
       </c>
       <c r="B19" s="39" t="n">
         <f aca="false">IF(K18="","",IF(K18&gt;$K$2,"",K18))</f>
-        <v>46341</v>
+        <v>46310</v>
       </c>
       <c r="C19" s="38" t="str">
         <f aca="false">IF(B19="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B19)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D19" s="40" t="str">
         <f aca="false">IF(B19="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -7652,7 +8535,7 @@
       <c r="I19" s="45"/>
       <c r="K19" s="27" t="n">
         <f aca="false">IF(B19="","",B19+MIN(MOD(הגדרות!$D$18-WEEKDAY(B19)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B19)-1,7)+1))</f>
-        <v>46345</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7662,11 +8545,11 @@
       </c>
       <c r="B20" s="39" t="n">
         <f aca="false">IF(K19="","",IF(K19&gt;$K$2,"",K19))</f>
-        <v>46345</v>
+        <v>46313</v>
       </c>
       <c r="C20" s="38" t="str">
         <f aca="false">IF(B20="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B20)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D20" s="40" t="str">
         <f aca="false">IF(B20="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -7687,7 +8570,7 @@
       <c r="I20" s="45"/>
       <c r="K20" s="27" t="n">
         <f aca="false">IF(B20="","",B20+MIN(MOD(הגדרות!$D$18-WEEKDAY(B20)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B20)-1,7)+1))</f>
-        <v>46348</v>
+        <v>46317</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7697,11 +8580,11 @@
       </c>
       <c r="B21" s="39" t="n">
         <f aca="false">IF(K20="","",IF(K20&gt;$K$2,"",K20))</f>
-        <v>46348</v>
+        <v>46317</v>
       </c>
       <c r="C21" s="38" t="str">
         <f aca="false">IF(B21="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B21)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D21" s="40" t="str">
         <f aca="false">IF(B21="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -7722,7 +8605,7 @@
       <c r="I21" s="45"/>
       <c r="K21" s="27" t="n">
         <f aca="false">IF(B21="","",B21+MIN(MOD(הגדרות!$D$18-WEEKDAY(B21)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B21)-1,7)+1))</f>
-        <v>46352</v>
+        <v>46320</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7732,11 +8615,11 @@
       </c>
       <c r="B22" s="39" t="n">
         <f aca="false">IF(K21="","",IF(K21&gt;$K$2,"",K21))</f>
-        <v>46352</v>
+        <v>46320</v>
       </c>
       <c r="C22" s="38" t="str">
         <f aca="false">IF(B22="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B22)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D22" s="40" t="str">
         <f aca="false">IF(B22="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -7757,7 +8640,7 @@
       <c r="I22" s="45"/>
       <c r="K22" s="27" t="n">
         <f aca="false">IF(B22="","",B22+MIN(MOD(הגדרות!$D$18-WEEKDAY(B22)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B22)-1,7)+1))</f>
-        <v>46355</v>
+        <v>46324</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7767,11 +8650,11 @@
       </c>
       <c r="B23" s="39" t="n">
         <f aca="false">IF(K22="","",IF(K22&gt;$K$2,"",K22))</f>
-        <v>46355</v>
+        <v>46324</v>
       </c>
       <c r="C23" s="38" t="str">
         <f aca="false">IF(B23="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B23)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D23" s="40" t="str">
         <f aca="false">IF(B23="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -7792,7 +8675,7 @@
       <c r="I23" s="45"/>
       <c r="K23" s="27" t="n">
         <f aca="false">IF(B23="","",B23+MIN(MOD(הגדרות!$D$18-WEEKDAY(B23)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B23)-1,7)+1))</f>
-        <v>46359</v>
+        <v>46327</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8109,13 +8992,13 @@
       <c r="I1" s="26"/>
       <c r="K1" s="27" t="n">
         <f aca="false">DATE(YEAR($H$11),MONTH($H$11),1)</f>
-        <v>46357</v>
+        <v>46327</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="str">
         <f aca="false">הגדרות!$C$17&amp;" · "&amp;CHOOSE(MONTH($K$1),"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר")&amp;" "&amp;YEAR($K$1)</f>
-        <v>הדרכת שיקום · דצמבר 2026</v>
+        <v>הדרכת שיקום · נובמבר 2026</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -8127,7 +9010,7 @@
       <c r="I2" s="28"/>
       <c r="K2" s="27" t="n">
         <f aca="false">EOMONTH($K$1,0)</f>
-        <v>46387</v>
+        <v>46356</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -8235,7 +9118,7 @@
       <c r="B11" s="30"/>
       <c r="C11" s="31" t="str">
         <f aca="false">YEAR($K$1)&amp;"-"&amp;TEXT(MONTH($K$1),"00")</f>
-        <v>2026-12</v>
+        <v>2026-11</v>
       </c>
       <c r="D11" s="31"/>
       <c r="F11" s="30" t="s">
@@ -8243,7 +9126,7 @@
       </c>
       <c r="G11" s="30"/>
       <c r="H11" s="32" t="n">
-        <v>46357</v>
+        <v>46327</v>
       </c>
       <c r="I11" s="32"/>
     </row>
@@ -8254,7 +9137,7 @@
       <c r="B12" s="30"/>
       <c r="C12" s="33" t="n">
         <f aca="false">$K$2</f>
-        <v>46387</v>
+        <v>46356</v>
       </c>
       <c r="D12" s="33"/>
       <c r="F12" s="30" t="s">
@@ -8318,11 +9201,11 @@
       </c>
       <c r="B15" s="39" t="n">
         <f aca="false">$K$1+MIN(MOD(הגדרות!$D$18-WEEKDAY($K$1),7),MOD(הגדרות!$D$19-WEEKDAY($K$1),7))</f>
-        <v>46359</v>
+        <v>46327</v>
       </c>
       <c r="C15" s="38" t="str">
         <f aca="false">IF(B15="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B15)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D15" s="40" t="str">
         <f aca="false">IF(B15="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -8343,7 +9226,7 @@
       <c r="I15" s="45"/>
       <c r="K15" s="27" t="n">
         <f aca="false">IF(B15="","",B15+MIN(MOD(הגדרות!$D$18-WEEKDAY(B15)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B15)-1,7)+1))</f>
-        <v>46362</v>
+        <v>46331</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8353,11 +9236,11 @@
       </c>
       <c r="B16" s="39" t="n">
         <f aca="false">IF(K15="","",IF(K15&gt;$K$2,"",K15))</f>
-        <v>46362</v>
+        <v>46331</v>
       </c>
       <c r="C16" s="38" t="str">
         <f aca="false">IF(B16="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B16)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D16" s="40" t="str">
         <f aca="false">IF(B16="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -8378,7 +9261,7 @@
       <c r="I16" s="45"/>
       <c r="K16" s="27" t="n">
         <f aca="false">IF(B16="","",B16+MIN(MOD(הגדרות!$D$18-WEEKDAY(B16)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B16)-1,7)+1))</f>
-        <v>46366</v>
+        <v>46334</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8388,11 +9271,11 @@
       </c>
       <c r="B17" s="39" t="n">
         <f aca="false">IF(K16="","",IF(K16&gt;$K$2,"",K16))</f>
-        <v>46366</v>
+        <v>46334</v>
       </c>
       <c r="C17" s="38" t="str">
         <f aca="false">IF(B17="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B17)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D17" s="40" t="str">
         <f aca="false">IF(B17="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -8413,7 +9296,7 @@
       <c r="I17" s="45"/>
       <c r="K17" s="27" t="n">
         <f aca="false">IF(B17="","",B17+MIN(MOD(הגדרות!$D$18-WEEKDAY(B17)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B17)-1,7)+1))</f>
-        <v>46369</v>
+        <v>46338</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8423,11 +9306,11 @@
       </c>
       <c r="B18" s="39" t="n">
         <f aca="false">IF(K17="","",IF(K17&gt;$K$2,"",K17))</f>
-        <v>46369</v>
+        <v>46338</v>
       </c>
       <c r="C18" s="38" t="str">
         <f aca="false">IF(B18="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B18)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D18" s="40" t="str">
         <f aca="false">IF(B18="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -8448,7 +9331,7 @@
       <c r="I18" s="45"/>
       <c r="K18" s="27" t="n">
         <f aca="false">IF(B18="","",B18+MIN(MOD(הגדרות!$D$18-WEEKDAY(B18)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B18)-1,7)+1))</f>
-        <v>46373</v>
+        <v>46341</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8458,11 +9341,11 @@
       </c>
       <c r="B19" s="39" t="n">
         <f aca="false">IF(K18="","",IF(K18&gt;$K$2,"",K18))</f>
-        <v>46373</v>
+        <v>46341</v>
       </c>
       <c r="C19" s="38" t="str">
         <f aca="false">IF(B19="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B19)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D19" s="40" t="str">
         <f aca="false">IF(B19="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -8483,7 +9366,7 @@
       <c r="I19" s="45"/>
       <c r="K19" s="27" t="n">
         <f aca="false">IF(B19="","",B19+MIN(MOD(הגדרות!$D$18-WEEKDAY(B19)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B19)-1,7)+1))</f>
-        <v>46376</v>
+        <v>46345</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8493,11 +9376,11 @@
       </c>
       <c r="B20" s="39" t="n">
         <f aca="false">IF(K19="","",IF(K19&gt;$K$2,"",K19))</f>
-        <v>46376</v>
+        <v>46345</v>
       </c>
       <c r="C20" s="38" t="str">
         <f aca="false">IF(B20="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B20)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D20" s="40" t="str">
         <f aca="false">IF(B20="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -8518,7 +9401,7 @@
       <c r="I20" s="45"/>
       <c r="K20" s="27" t="n">
         <f aca="false">IF(B20="","",B20+MIN(MOD(הגדרות!$D$18-WEEKDAY(B20)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B20)-1,7)+1))</f>
-        <v>46380</v>
+        <v>46348</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8528,11 +9411,11 @@
       </c>
       <c r="B21" s="39" t="n">
         <f aca="false">IF(K20="","",IF(K20&gt;$K$2,"",K20))</f>
-        <v>46380</v>
+        <v>46348</v>
       </c>
       <c r="C21" s="38" t="str">
         <f aca="false">IF(B21="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B21)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D21" s="40" t="str">
         <f aca="false">IF(B21="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -8553,7 +9436,7 @@
       <c r="I21" s="45"/>
       <c r="K21" s="27" t="n">
         <f aca="false">IF(B21="","",B21+MIN(MOD(הגדרות!$D$18-WEEKDAY(B21)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B21)-1,7)+1))</f>
-        <v>46383</v>
+        <v>46352</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8563,11 +9446,11 @@
       </c>
       <c r="B22" s="39" t="n">
         <f aca="false">IF(K21="","",IF(K21&gt;$K$2,"",K21))</f>
-        <v>46383</v>
+        <v>46352</v>
       </c>
       <c r="C22" s="38" t="str">
         <f aca="false">IF(B22="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B22)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D22" s="40" t="str">
         <f aca="false">IF(B22="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -8588,7 +9471,7 @@
       <c r="I22" s="45"/>
       <c r="K22" s="27" t="n">
         <f aca="false">IF(B22="","",B22+MIN(MOD(הגדרות!$D$18-WEEKDAY(B22)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B22)-1,7)+1))</f>
-        <v>46387</v>
+        <v>46355</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8598,11 +9481,11 @@
       </c>
       <c r="B23" s="39" t="n">
         <f aca="false">IF(K22="","",IF(K22&gt;$K$2,"",K22))</f>
-        <v>46387</v>
+        <v>46355</v>
       </c>
       <c r="C23" s="38" t="str">
         <f aca="false">IF(B23="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B23)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D23" s="40" t="str">
         <f aca="false">IF(B23="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -8623,7 +9506,7 @@
       <c r="I23" s="45"/>
       <c r="K23" s="27" t="n">
         <f aca="false">IF(B23="","",B23+MIN(MOD(הגדרות!$D$18-WEEKDAY(B23)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B23)-1,7)+1))</f>
-        <v>46390</v>
+        <v>46359</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8940,13 +9823,13 @@
       <c r="I1" s="26"/>
       <c r="K1" s="27" t="n">
         <f aca="false">DATE(YEAR($H$11),MONTH($H$11),1)</f>
-        <v>46388</v>
+        <v>46357</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="str">
         <f aca="false">הגדרות!$C$17&amp;" · "&amp;CHOOSE(MONTH($K$1),"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר")&amp;" "&amp;YEAR($K$1)</f>
-        <v>הדרכת שיקום · ינואר 2027</v>
+        <v>הדרכת שיקום · דצמבר 2026</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -8958,7 +9841,7 @@
       <c r="I2" s="28"/>
       <c r="K2" s="27" t="n">
         <f aca="false">EOMONTH($K$1,0)</f>
-        <v>46418</v>
+        <v>46387</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -9066,7 +9949,7 @@
       <c r="B11" s="30"/>
       <c r="C11" s="31" t="str">
         <f aca="false">YEAR($K$1)&amp;"-"&amp;TEXT(MONTH($K$1),"00")</f>
-        <v>2027-01</v>
+        <v>2026-12</v>
       </c>
       <c r="D11" s="31"/>
       <c r="F11" s="30" t="s">
@@ -9074,7 +9957,7 @@
       </c>
       <c r="G11" s="30"/>
       <c r="H11" s="32" t="n">
-        <v>46388</v>
+        <v>46357</v>
       </c>
       <c r="I11" s="32"/>
     </row>
@@ -9085,7 +9968,7 @@
       <c r="B12" s="30"/>
       <c r="C12" s="33" t="n">
         <f aca="false">$K$2</f>
-        <v>46418</v>
+        <v>46387</v>
       </c>
       <c r="D12" s="33"/>
       <c r="F12" s="30" t="s">
@@ -9149,11 +10032,11 @@
       </c>
       <c r="B15" s="39" t="n">
         <f aca="false">$K$1+MIN(MOD(הגדרות!$D$18-WEEKDAY($K$1),7),MOD(הגדרות!$D$19-WEEKDAY($K$1),7))</f>
-        <v>46390</v>
+        <v>46359</v>
       </c>
       <c r="C15" s="38" t="str">
         <f aca="false">IF(B15="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B15)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D15" s="40" t="str">
         <f aca="false">IF(B15="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -9174,7 +10057,7 @@
       <c r="I15" s="45"/>
       <c r="K15" s="27" t="n">
         <f aca="false">IF(B15="","",B15+MIN(MOD(הגדרות!$D$18-WEEKDAY(B15)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B15)-1,7)+1))</f>
-        <v>46394</v>
+        <v>46362</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9184,11 +10067,11 @@
       </c>
       <c r="B16" s="39" t="n">
         <f aca="false">IF(K15="","",IF(K15&gt;$K$2,"",K15))</f>
-        <v>46394</v>
+        <v>46362</v>
       </c>
       <c r="C16" s="38" t="str">
         <f aca="false">IF(B16="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B16)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D16" s="40" t="str">
         <f aca="false">IF(B16="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -9209,7 +10092,7 @@
       <c r="I16" s="45"/>
       <c r="K16" s="27" t="n">
         <f aca="false">IF(B16="","",B16+MIN(MOD(הגדרות!$D$18-WEEKDAY(B16)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B16)-1,7)+1))</f>
-        <v>46397</v>
+        <v>46366</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9219,11 +10102,11 @@
       </c>
       <c r="B17" s="39" t="n">
         <f aca="false">IF(K16="","",IF(K16&gt;$K$2,"",K16))</f>
-        <v>46397</v>
+        <v>46366</v>
       </c>
       <c r="C17" s="38" t="str">
         <f aca="false">IF(B17="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B17)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D17" s="40" t="str">
         <f aca="false">IF(B17="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -9244,7 +10127,7 @@
       <c r="I17" s="45"/>
       <c r="K17" s="27" t="n">
         <f aca="false">IF(B17="","",B17+MIN(MOD(הגדרות!$D$18-WEEKDAY(B17)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B17)-1,7)+1))</f>
-        <v>46401</v>
+        <v>46369</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9254,11 +10137,11 @@
       </c>
       <c r="B18" s="39" t="n">
         <f aca="false">IF(K17="","",IF(K17&gt;$K$2,"",K17))</f>
-        <v>46401</v>
+        <v>46369</v>
       </c>
       <c r="C18" s="38" t="str">
         <f aca="false">IF(B18="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B18)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D18" s="40" t="str">
         <f aca="false">IF(B18="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -9279,7 +10162,7 @@
       <c r="I18" s="45"/>
       <c r="K18" s="27" t="n">
         <f aca="false">IF(B18="","",B18+MIN(MOD(הגדרות!$D$18-WEEKDAY(B18)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B18)-1,7)+1))</f>
-        <v>46404</v>
+        <v>46373</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9289,11 +10172,11 @@
       </c>
       <c r="B19" s="39" t="n">
         <f aca="false">IF(K18="","",IF(K18&gt;$K$2,"",K18))</f>
-        <v>46404</v>
+        <v>46373</v>
       </c>
       <c r="C19" s="38" t="str">
         <f aca="false">IF(B19="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B19)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D19" s="40" t="str">
         <f aca="false">IF(B19="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -9314,7 +10197,7 @@
       <c r="I19" s="45"/>
       <c r="K19" s="27" t="n">
         <f aca="false">IF(B19="","",B19+MIN(MOD(הגדרות!$D$18-WEEKDAY(B19)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B19)-1,7)+1))</f>
-        <v>46408</v>
+        <v>46376</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9324,11 +10207,11 @@
       </c>
       <c r="B20" s="39" t="n">
         <f aca="false">IF(K19="","",IF(K19&gt;$K$2,"",K19))</f>
-        <v>46408</v>
+        <v>46376</v>
       </c>
       <c r="C20" s="38" t="str">
         <f aca="false">IF(B20="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B20)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D20" s="40" t="str">
         <f aca="false">IF(B20="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -9349,7 +10232,7 @@
       <c r="I20" s="45"/>
       <c r="K20" s="27" t="n">
         <f aca="false">IF(B20="","",B20+MIN(MOD(הגדרות!$D$18-WEEKDAY(B20)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B20)-1,7)+1))</f>
-        <v>46411</v>
+        <v>46380</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9359,11 +10242,11 @@
       </c>
       <c r="B21" s="39" t="n">
         <f aca="false">IF(K20="","",IF(K20&gt;$K$2,"",K20))</f>
-        <v>46411</v>
+        <v>46380</v>
       </c>
       <c r="C21" s="38" t="str">
         <f aca="false">IF(B21="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B21)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D21" s="40" t="str">
         <f aca="false">IF(B21="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -9384,7 +10267,7 @@
       <c r="I21" s="45"/>
       <c r="K21" s="27" t="n">
         <f aca="false">IF(B21="","",B21+MIN(MOD(הגדרות!$D$18-WEEKDAY(B21)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B21)-1,7)+1))</f>
-        <v>46415</v>
+        <v>46383</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9394,11 +10277,11 @@
       </c>
       <c r="B22" s="39" t="n">
         <f aca="false">IF(K21="","",IF(K21&gt;$K$2,"",K21))</f>
-        <v>46415</v>
+        <v>46383</v>
       </c>
       <c r="C22" s="38" t="str">
         <f aca="false">IF(B22="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B22)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D22" s="40" t="str">
         <f aca="false">IF(B22="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -9419,7 +10302,7 @@
       <c r="I22" s="45"/>
       <c r="K22" s="27" t="n">
         <f aca="false">IF(B22="","",B22+MIN(MOD(הגדרות!$D$18-WEEKDAY(B22)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B22)-1,7)+1))</f>
-        <v>46418</v>
+        <v>46387</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9429,11 +10312,11 @@
       </c>
       <c r="B23" s="39" t="n">
         <f aca="false">IF(K22="","",IF(K22&gt;$K$2,"",K22))</f>
-        <v>46418</v>
+        <v>46387</v>
       </c>
       <c r="C23" s="38" t="str">
         <f aca="false">IF(B23="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B23)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D23" s="40" t="str">
         <f aca="false">IF(B23="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -9454,7 +10337,7 @@
       <c r="I23" s="45"/>
       <c r="K23" s="27" t="n">
         <f aca="false">IF(B23="","",B23+MIN(MOD(הגדרות!$D$18-WEEKDAY(B23)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B23)-1,7)+1))</f>
-        <v>46422</v>
+        <v>46390</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9771,13 +10654,13 @@
       <c r="I1" s="26"/>
       <c r="K1" s="27" t="n">
         <f aca="false">DATE(YEAR($H$11),MONTH($H$11),1)</f>
-        <v>46419</v>
+        <v>46388</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="str">
         <f aca="false">הגדרות!$C$17&amp;" · "&amp;CHOOSE(MONTH($K$1),"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר")&amp;" "&amp;YEAR($K$1)</f>
-        <v>הדרכת שיקום · פברואר 2027</v>
+        <v>הדרכת שיקום · ינואר 2027</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -9789,7 +10672,7 @@
       <c r="I2" s="28"/>
       <c r="K2" s="27" t="n">
         <f aca="false">EOMONTH($K$1,0)</f>
-        <v>46446</v>
+        <v>46418</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -9897,7 +10780,7 @@
       <c r="B11" s="30"/>
       <c r="C11" s="31" t="str">
         <f aca="false">YEAR($K$1)&amp;"-"&amp;TEXT(MONTH($K$1),"00")</f>
-        <v>2027-02</v>
+        <v>2027-01</v>
       </c>
       <c r="D11" s="31"/>
       <c r="F11" s="30" t="s">
@@ -9905,7 +10788,7 @@
       </c>
       <c r="G11" s="30"/>
       <c r="H11" s="32" t="n">
-        <v>46419</v>
+        <v>46388</v>
       </c>
       <c r="I11" s="32"/>
     </row>
@@ -9916,7 +10799,7 @@
       <c r="B12" s="30"/>
       <c r="C12" s="33" t="n">
         <f aca="false">$K$2</f>
-        <v>46446</v>
+        <v>46418</v>
       </c>
       <c r="D12" s="33"/>
       <c r="F12" s="30" t="s">
@@ -9980,11 +10863,11 @@
       </c>
       <c r="B15" s="39" t="n">
         <f aca="false">$K$1+MIN(MOD(הגדרות!$D$18-WEEKDAY($K$1),7),MOD(הגדרות!$D$19-WEEKDAY($K$1),7))</f>
-        <v>46422</v>
+        <v>46390</v>
       </c>
       <c r="C15" s="38" t="str">
         <f aca="false">IF(B15="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B15)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D15" s="40" t="str">
         <f aca="false">IF(B15="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -10005,7 +10888,7 @@
       <c r="I15" s="45"/>
       <c r="K15" s="27" t="n">
         <f aca="false">IF(B15="","",B15+MIN(MOD(הגדרות!$D$18-WEEKDAY(B15)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B15)-1,7)+1))</f>
-        <v>46425</v>
+        <v>46394</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10015,11 +10898,11 @@
       </c>
       <c r="B16" s="39" t="n">
         <f aca="false">IF(K15="","",IF(K15&gt;$K$2,"",K15))</f>
-        <v>46425</v>
+        <v>46394</v>
       </c>
       <c r="C16" s="38" t="str">
         <f aca="false">IF(B16="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B16)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D16" s="40" t="str">
         <f aca="false">IF(B16="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -10040,7 +10923,7 @@
       <c r="I16" s="45"/>
       <c r="K16" s="27" t="n">
         <f aca="false">IF(B16="","",B16+MIN(MOD(הגדרות!$D$18-WEEKDAY(B16)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B16)-1,7)+1))</f>
-        <v>46429</v>
+        <v>46397</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10050,11 +10933,11 @@
       </c>
       <c r="B17" s="39" t="n">
         <f aca="false">IF(K16="","",IF(K16&gt;$K$2,"",K16))</f>
-        <v>46429</v>
+        <v>46397</v>
       </c>
       <c r="C17" s="38" t="str">
         <f aca="false">IF(B17="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B17)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D17" s="40" t="str">
         <f aca="false">IF(B17="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -10075,7 +10958,7 @@
       <c r="I17" s="45"/>
       <c r="K17" s="27" t="n">
         <f aca="false">IF(B17="","",B17+MIN(MOD(הגדרות!$D$18-WEEKDAY(B17)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B17)-1,7)+1))</f>
-        <v>46432</v>
+        <v>46401</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10085,11 +10968,11 @@
       </c>
       <c r="B18" s="39" t="n">
         <f aca="false">IF(K17="","",IF(K17&gt;$K$2,"",K17))</f>
-        <v>46432</v>
+        <v>46401</v>
       </c>
       <c r="C18" s="38" t="str">
         <f aca="false">IF(B18="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B18)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D18" s="40" t="str">
         <f aca="false">IF(B18="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -10110,7 +10993,7 @@
       <c r="I18" s="45"/>
       <c r="K18" s="27" t="n">
         <f aca="false">IF(B18="","",B18+MIN(MOD(הגדרות!$D$18-WEEKDAY(B18)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B18)-1,7)+1))</f>
-        <v>46436</v>
+        <v>46404</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10120,11 +11003,11 @@
       </c>
       <c r="B19" s="39" t="n">
         <f aca="false">IF(K18="","",IF(K18&gt;$K$2,"",K18))</f>
-        <v>46436</v>
+        <v>46404</v>
       </c>
       <c r="C19" s="38" t="str">
         <f aca="false">IF(B19="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B19)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D19" s="40" t="str">
         <f aca="false">IF(B19="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -10145,7 +11028,7 @@
       <c r="I19" s="45"/>
       <c r="K19" s="27" t="n">
         <f aca="false">IF(B19="","",B19+MIN(MOD(הגדרות!$D$18-WEEKDAY(B19)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B19)-1,7)+1))</f>
-        <v>46439</v>
+        <v>46408</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10155,11 +11038,11 @@
       </c>
       <c r="B20" s="39" t="n">
         <f aca="false">IF(K19="","",IF(K19&gt;$K$2,"",K19))</f>
-        <v>46439</v>
+        <v>46408</v>
       </c>
       <c r="C20" s="38" t="str">
         <f aca="false">IF(B20="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B20)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D20" s="40" t="str">
         <f aca="false">IF(B20="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -10180,7 +11063,7 @@
       <c r="I20" s="45"/>
       <c r="K20" s="27" t="n">
         <f aca="false">IF(B20="","",B20+MIN(MOD(הגדרות!$D$18-WEEKDAY(B20)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B20)-1,7)+1))</f>
-        <v>46443</v>
+        <v>46411</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10190,11 +11073,11 @@
       </c>
       <c r="B21" s="39" t="n">
         <f aca="false">IF(K20="","",IF(K20&gt;$K$2,"",K20))</f>
-        <v>46443</v>
+        <v>46411</v>
       </c>
       <c r="C21" s="38" t="str">
         <f aca="false">IF(B21="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B21)))</f>
-        <v>חמישי</v>
+        <v>ראשון</v>
       </c>
       <c r="D21" s="40" t="str">
         <f aca="false">IF(B21="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -10215,7 +11098,7 @@
       <c r="I21" s="45"/>
       <c r="K21" s="27" t="n">
         <f aca="false">IF(B21="","",B21+MIN(MOD(הגדרות!$D$18-WEEKDAY(B21)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B21)-1,7)+1))</f>
-        <v>46446</v>
+        <v>46415</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10225,11 +11108,11 @@
       </c>
       <c r="B22" s="39" t="n">
         <f aca="false">IF(K21="","",IF(K21&gt;$K$2,"",K21))</f>
-        <v>46446</v>
+        <v>46415</v>
       </c>
       <c r="C22" s="38" t="str">
         <f aca="false">IF(B22="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B22)))</f>
-        <v>ראשון</v>
+        <v>חמישי</v>
       </c>
       <c r="D22" s="40" t="str">
         <f aca="false">IF(B22="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
@@ -10250,42 +11133,42 @@
       <c r="I22" s="45"/>
       <c r="K22" s="27" t="n">
         <f aca="false">IF(B22="","",B22+MIN(MOD(הגדרות!$D$18-WEEKDAY(B22)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B22)-1,7)+1))</f>
-        <v>46450</v>
+        <v>46418</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="38" t="str">
+      <c r="A23" s="38" t="n">
         <f aca="false">IF(B23="","",ROW()-14)</f>
-        <v/>
-      </c>
-      <c r="B23" s="39" t="str">
+        <v>9</v>
+      </c>
+      <c r="B23" s="39" t="n">
         <f aca="false">IF(K22="","",IF(K22&gt;$K$2,"",K22))</f>
-        <v/>
+        <v>46418</v>
       </c>
       <c r="C23" s="38" t="str">
         <f aca="false">IF(B23="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B23)))</f>
-        <v/>
+        <v>ראשון</v>
       </c>
       <c r="D23" s="40" t="str">
         <f aca="false">IF(B23="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
-        <v/>
+        <v>הדרכה 09:00–12:30</v>
       </c>
       <c r="E23" s="41" t="s">
         <v>83</v>
       </c>
-      <c r="F23" s="42" t="str">
+      <c r="F23" s="42" t="n">
         <f aca="false">IF(B23="","",IF(E23="לא",0,הגדרות!$C$22))</f>
-        <v/>
-      </c>
-      <c r="G23" s="43" t="str">
+        <v>3.5</v>
+      </c>
+      <c r="G23" s="43" t="n">
         <f aca="false">IF(B23="","",F23*הגדרות!$C$24)</f>
-        <v/>
+        <v>175</v>
       </c>
       <c r="H23" s="44"/>
       <c r="I23" s="45"/>
-      <c r="K23" s="27" t="str">
+      <c r="K23" s="27" t="n">
         <f aca="false">IF(B23="","",B23+MIN(MOD(הגדרות!$D$18-WEEKDAY(B23)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B23)-1,7)+1))</f>
-        <v/>
+        <v>46422</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10326,7 +11209,7 @@
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="38" t="n">
         <f aca="false">COUNT($B$15:$B$24)+1</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B25" s="46"/>
       <c r="C25" s="38" t="str">
@@ -10361,11 +11244,11 @@
       <c r="E26" s="47"/>
       <c r="F26" s="48" t="n">
         <f aca="false">SUM(F15:F25)</f>
-        <v>29</v>
+        <v>32.5</v>
       </c>
       <c r="G26" s="49" t="n">
         <f aca="false">SUM(G15:G25)</f>
-        <v>1450</v>
+        <v>1625</v>
       </c>
       <c r="H26" s="47"/>
       <c r="I26" s="49" t="n">
@@ -10387,7 +11270,7 @@
       <c r="H28" s="40"/>
       <c r="I28" s="42" t="n">
         <f aca="false">F26</f>
-        <v>29</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10401,13 +11284,13 @@
       <c r="E29" s="51"/>
       <c r="F29" s="40" t="str">
         <f aca="false">"הדרכת שיקום ("&amp;TEXT(F26,"0.0")&amp;" שעות × "&amp;הגדרות!$C$24&amp;" ₪)"</f>
-        <v>הדרכת שיקום (29.0 שעות × 50 ₪)</v>
+        <v>הדרכת שיקום (32.5 שעות × 50 ₪)</v>
       </c>
       <c r="G29" s="40"/>
       <c r="H29" s="40"/>
       <c r="I29" s="43" t="n">
         <f aca="false">G26</f>
-        <v>1450</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10445,7 +11328,7 @@
       <c r="H31" s="52"/>
       <c r="I31" s="53" t="n">
         <f aca="false">I29+I30</f>
-        <v>1450</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10465,7 +11348,7 @@
       <c r="H32" s="40"/>
       <c r="I32" s="43" t="n">
         <f aca="false">ROUND(I31*הגדרות!$C$25,2)</f>
-        <v>261</v>
+        <v>292.5</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10476,7 +11359,7 @@
       <c r="H33" s="54"/>
       <c r="I33" s="55" t="n">
         <f aca="false">I31+I32</f>
-        <v>1711</v>
+        <v>1917.5</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10602,13 +11485,13 @@
       <c r="I1" s="26"/>
       <c r="K1" s="27" t="n">
         <f aca="false">DATE(YEAR($H$11),MONTH($H$11),1)</f>
-        <v>46447</v>
+        <v>46419</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="str">
         <f aca="false">הגדרות!$C$17&amp;" · "&amp;CHOOSE(MONTH($K$1),"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר")&amp;" "&amp;YEAR($K$1)</f>
-        <v>הדרכת שיקום · מרץ 2027</v>
+        <v>הדרכת שיקום · פברואר 2027</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -10620,7 +11503,7 @@
       <c r="I2" s="28"/>
       <c r="K2" s="27" t="n">
         <f aca="false">EOMONTH($K$1,0)</f>
-        <v>46477</v>
+        <v>46446</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -10728,7 +11611,7 @@
       <c r="B11" s="30"/>
       <c r="C11" s="31" t="str">
         <f aca="false">YEAR($K$1)&amp;"-"&amp;TEXT(MONTH($K$1),"00")</f>
-        <v>2027-03</v>
+        <v>2027-02</v>
       </c>
       <c r="D11" s="31"/>
       <c r="F11" s="30" t="s">
@@ -10736,7 +11619,7 @@
       </c>
       <c r="G11" s="30"/>
       <c r="H11" s="32" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="I11" s="32"/>
     </row>
@@ -10747,7 +11630,7 @@
       <c r="B12" s="30"/>
       <c r="C12" s="33" t="n">
         <f aca="false">$K$2</f>
-        <v>46477</v>
+        <v>46446</v>
       </c>
       <c r="D12" s="33"/>
       <c r="F12" s="30" t="s">
@@ -10811,7 +11694,7 @@
       </c>
       <c r="B15" s="39" t="n">
         <f aca="false">$K$1+MIN(MOD(הגדרות!$D$18-WEEKDAY($K$1),7),MOD(הגדרות!$D$19-WEEKDAY($K$1),7))</f>
-        <v>46450</v>
+        <v>46422</v>
       </c>
       <c r="C15" s="38" t="str">
         <f aca="false">IF(B15="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B15)))</f>
@@ -10836,7 +11719,7 @@
       <c r="I15" s="45"/>
       <c r="K15" s="27" t="n">
         <f aca="false">IF(B15="","",B15+MIN(MOD(הגדרות!$D$18-WEEKDAY(B15)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B15)-1,7)+1))</f>
-        <v>46453</v>
+        <v>46425</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10846,7 +11729,7 @@
       </c>
       <c r="B16" s="39" t="n">
         <f aca="false">IF(K15="","",IF(K15&gt;$K$2,"",K15))</f>
-        <v>46453</v>
+        <v>46425</v>
       </c>
       <c r="C16" s="38" t="str">
         <f aca="false">IF(B16="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B16)))</f>
@@ -10871,7 +11754,7 @@
       <c r="I16" s="45"/>
       <c r="K16" s="27" t="n">
         <f aca="false">IF(B16="","",B16+MIN(MOD(הגדרות!$D$18-WEEKDAY(B16)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B16)-1,7)+1))</f>
-        <v>46457</v>
+        <v>46429</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10881,7 +11764,7 @@
       </c>
       <c r="B17" s="39" t="n">
         <f aca="false">IF(K16="","",IF(K16&gt;$K$2,"",K16))</f>
-        <v>46457</v>
+        <v>46429</v>
       </c>
       <c r="C17" s="38" t="str">
         <f aca="false">IF(B17="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B17)))</f>
@@ -10906,7 +11789,7 @@
       <c r="I17" s="45"/>
       <c r="K17" s="27" t="n">
         <f aca="false">IF(B17="","",B17+MIN(MOD(הגדרות!$D$18-WEEKDAY(B17)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B17)-1,7)+1))</f>
-        <v>46460</v>
+        <v>46432</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10916,7 +11799,7 @@
       </c>
       <c r="B18" s="39" t="n">
         <f aca="false">IF(K17="","",IF(K17&gt;$K$2,"",K17))</f>
-        <v>46460</v>
+        <v>46432</v>
       </c>
       <c r="C18" s="38" t="str">
         <f aca="false">IF(B18="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B18)))</f>
@@ -10941,7 +11824,7 @@
       <c r="I18" s="45"/>
       <c r="K18" s="27" t="n">
         <f aca="false">IF(B18="","",B18+MIN(MOD(הגדרות!$D$18-WEEKDAY(B18)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B18)-1,7)+1))</f>
-        <v>46464</v>
+        <v>46436</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10951,7 +11834,7 @@
       </c>
       <c r="B19" s="39" t="n">
         <f aca="false">IF(K18="","",IF(K18&gt;$K$2,"",K18))</f>
-        <v>46464</v>
+        <v>46436</v>
       </c>
       <c r="C19" s="38" t="str">
         <f aca="false">IF(B19="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B19)))</f>
@@ -10976,7 +11859,7 @@
       <c r="I19" s="45"/>
       <c r="K19" s="27" t="n">
         <f aca="false">IF(B19="","",B19+MIN(MOD(הגדרות!$D$18-WEEKDAY(B19)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B19)-1,7)+1))</f>
-        <v>46467</v>
+        <v>46439</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10986,7 +11869,7 @@
       </c>
       <c r="B20" s="39" t="n">
         <f aca="false">IF(K19="","",IF(K19&gt;$K$2,"",K19))</f>
-        <v>46467</v>
+        <v>46439</v>
       </c>
       <c r="C20" s="38" t="str">
         <f aca="false">IF(B20="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B20)))</f>
@@ -11011,7 +11894,7 @@
       <c r="I20" s="45"/>
       <c r="K20" s="27" t="n">
         <f aca="false">IF(B20="","",B20+MIN(MOD(הגדרות!$D$18-WEEKDAY(B20)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B20)-1,7)+1))</f>
-        <v>46471</v>
+        <v>46443</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11021,7 +11904,7 @@
       </c>
       <c r="B21" s="39" t="n">
         <f aca="false">IF(K20="","",IF(K20&gt;$K$2,"",K20))</f>
-        <v>46471</v>
+        <v>46443</v>
       </c>
       <c r="C21" s="38" t="str">
         <f aca="false">IF(B21="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B21)))</f>
@@ -11046,7 +11929,7 @@
       <c r="I21" s="45"/>
       <c r="K21" s="27" t="n">
         <f aca="false">IF(B21="","",B21+MIN(MOD(הגדרות!$D$18-WEEKDAY(B21)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B21)-1,7)+1))</f>
-        <v>46474</v>
+        <v>46446</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11056,7 +11939,7 @@
       </c>
       <c r="B22" s="39" t="n">
         <f aca="false">IF(K21="","",IF(K21&gt;$K$2,"",K21))</f>
-        <v>46474</v>
+        <v>46446</v>
       </c>
       <c r="C22" s="38" t="str">
         <f aca="false">IF(B22="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B22)))</f>
@@ -11081,7 +11964,7 @@
       <c r="I22" s="45"/>
       <c r="K22" s="27" t="n">
         <f aca="false">IF(B22="","",B22+MIN(MOD(הגדרות!$D$18-WEEKDAY(B22)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B22)-1,7)+1))</f>
-        <v>46478</v>
+        <v>46450</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11433,13 +12316,13 @@
       <c r="I1" s="26"/>
       <c r="K1" s="27" t="n">
         <f aca="false">DATE(YEAR($H$11),MONTH($H$11),1)</f>
-        <v>46478</v>
+        <v>46447</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="str">
         <f aca="false">הגדרות!$C$17&amp;" · "&amp;CHOOSE(MONTH($K$1),"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר")&amp;" "&amp;YEAR($K$1)</f>
-        <v>הדרכת שיקום · אפריל 2027</v>
+        <v>הדרכת שיקום · מרץ 2027</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -11451,7 +12334,7 @@
       <c r="I2" s="28"/>
       <c r="K2" s="27" t="n">
         <f aca="false">EOMONTH($K$1,0)</f>
-        <v>46507</v>
+        <v>46477</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -11559,7 +12442,7 @@
       <c r="B11" s="30"/>
       <c r="C11" s="31" t="str">
         <f aca="false">YEAR($K$1)&amp;"-"&amp;TEXT(MONTH($K$1),"00")</f>
-        <v>2027-04</v>
+        <v>2027-03</v>
       </c>
       <c r="D11" s="31"/>
       <c r="F11" s="30" t="s">
@@ -11567,7 +12450,7 @@
       </c>
       <c r="G11" s="30"/>
       <c r="H11" s="32" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="I11" s="32"/>
     </row>
@@ -11578,7 +12461,7 @@
       <c r="B12" s="30"/>
       <c r="C12" s="33" t="n">
         <f aca="false">$K$2</f>
-        <v>46507</v>
+        <v>46477</v>
       </c>
       <c r="D12" s="33"/>
       <c r="F12" s="30" t="s">
@@ -11642,7 +12525,7 @@
       </c>
       <c r="B15" s="39" t="n">
         <f aca="false">$K$1+MIN(MOD(הגדרות!$D$18-WEEKDAY($K$1),7),MOD(הגדרות!$D$19-WEEKDAY($K$1),7))</f>
-        <v>46478</v>
+        <v>46450</v>
       </c>
       <c r="C15" s="38" t="str">
         <f aca="false">IF(B15="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B15)))</f>
@@ -11667,7 +12550,7 @@
       <c r="I15" s="45"/>
       <c r="K15" s="27" t="n">
         <f aca="false">IF(B15="","",B15+MIN(MOD(הגדרות!$D$18-WEEKDAY(B15)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B15)-1,7)+1))</f>
-        <v>46481</v>
+        <v>46453</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11677,7 +12560,7 @@
       </c>
       <c r="B16" s="39" t="n">
         <f aca="false">IF(K15="","",IF(K15&gt;$K$2,"",K15))</f>
-        <v>46481</v>
+        <v>46453</v>
       </c>
       <c r="C16" s="38" t="str">
         <f aca="false">IF(B16="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B16)))</f>
@@ -11702,7 +12585,7 @@
       <c r="I16" s="45"/>
       <c r="K16" s="27" t="n">
         <f aca="false">IF(B16="","",B16+MIN(MOD(הגדרות!$D$18-WEEKDAY(B16)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B16)-1,7)+1))</f>
-        <v>46485</v>
+        <v>46457</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11712,7 +12595,7 @@
       </c>
       <c r="B17" s="39" t="n">
         <f aca="false">IF(K16="","",IF(K16&gt;$K$2,"",K16))</f>
-        <v>46485</v>
+        <v>46457</v>
       </c>
       <c r="C17" s="38" t="str">
         <f aca="false">IF(B17="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B17)))</f>
@@ -11737,7 +12620,7 @@
       <c r="I17" s="45"/>
       <c r="K17" s="27" t="n">
         <f aca="false">IF(B17="","",B17+MIN(MOD(הגדרות!$D$18-WEEKDAY(B17)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B17)-1,7)+1))</f>
-        <v>46488</v>
+        <v>46460</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11747,7 +12630,7 @@
       </c>
       <c r="B18" s="39" t="n">
         <f aca="false">IF(K17="","",IF(K17&gt;$K$2,"",K17))</f>
-        <v>46488</v>
+        <v>46460</v>
       </c>
       <c r="C18" s="38" t="str">
         <f aca="false">IF(B18="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B18)))</f>
@@ -11772,7 +12655,7 @@
       <c r="I18" s="45"/>
       <c r="K18" s="27" t="n">
         <f aca="false">IF(B18="","",B18+MIN(MOD(הגדרות!$D$18-WEEKDAY(B18)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B18)-1,7)+1))</f>
-        <v>46492</v>
+        <v>46464</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11782,7 +12665,7 @@
       </c>
       <c r="B19" s="39" t="n">
         <f aca="false">IF(K18="","",IF(K18&gt;$K$2,"",K18))</f>
-        <v>46492</v>
+        <v>46464</v>
       </c>
       <c r="C19" s="38" t="str">
         <f aca="false">IF(B19="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B19)))</f>
@@ -11807,7 +12690,7 @@
       <c r="I19" s="45"/>
       <c r="K19" s="27" t="n">
         <f aca="false">IF(B19="","",B19+MIN(MOD(הגדרות!$D$18-WEEKDAY(B19)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B19)-1,7)+1))</f>
-        <v>46495</v>
+        <v>46467</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11817,7 +12700,7 @@
       </c>
       <c r="B20" s="39" t="n">
         <f aca="false">IF(K19="","",IF(K19&gt;$K$2,"",K19))</f>
-        <v>46495</v>
+        <v>46467</v>
       </c>
       <c r="C20" s="38" t="str">
         <f aca="false">IF(B20="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B20)))</f>
@@ -11842,7 +12725,7 @@
       <c r="I20" s="45"/>
       <c r="K20" s="27" t="n">
         <f aca="false">IF(B20="","",B20+MIN(MOD(הגדרות!$D$18-WEEKDAY(B20)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B20)-1,7)+1))</f>
-        <v>46499</v>
+        <v>46471</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11852,7 +12735,7 @@
       </c>
       <c r="B21" s="39" t="n">
         <f aca="false">IF(K20="","",IF(K20&gt;$K$2,"",K20))</f>
-        <v>46499</v>
+        <v>46471</v>
       </c>
       <c r="C21" s="38" t="str">
         <f aca="false">IF(B21="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B21)))</f>
@@ -11877,7 +12760,7 @@
       <c r="I21" s="45"/>
       <c r="K21" s="27" t="n">
         <f aca="false">IF(B21="","",B21+MIN(MOD(הגדרות!$D$18-WEEKDAY(B21)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B21)-1,7)+1))</f>
-        <v>46502</v>
+        <v>46474</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11887,7 +12770,7 @@
       </c>
       <c r="B22" s="39" t="n">
         <f aca="false">IF(K21="","",IF(K21&gt;$K$2,"",K21))</f>
-        <v>46502</v>
+        <v>46474</v>
       </c>
       <c r="C22" s="38" t="str">
         <f aca="false">IF(B22="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B22)))</f>
@@ -11912,42 +12795,42 @@
       <c r="I22" s="45"/>
       <c r="K22" s="27" t="n">
         <f aca="false">IF(B22="","",B22+MIN(MOD(הגדרות!$D$18-WEEKDAY(B22)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B22)-1,7)+1))</f>
-        <v>46506</v>
+        <v>46478</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="38" t="n">
+      <c r="A23" s="38" t="str">
         <f aca="false">IF(B23="","",ROW()-14)</f>
-        <v>9</v>
-      </c>
-      <c r="B23" s="39" t="n">
+        <v/>
+      </c>
+      <c r="B23" s="39" t="str">
         <f aca="false">IF(K22="","",IF(K22&gt;$K$2,"",K22))</f>
-        <v>46506</v>
+        <v/>
       </c>
       <c r="C23" s="38" t="str">
         <f aca="false">IF(B23="","",INDEX(הגדרות!$F$5:$F$11,WEEKDAY(B23)))</f>
-        <v>חמישי</v>
+        <v/>
       </c>
       <c r="D23" s="40" t="str">
         <f aca="false">IF(B23="","","הדרכה "&amp;TEXT(HOUR(הגדרות!$C$20),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$20),"00")&amp;"–"&amp;TEXT(HOUR(הגדרות!$C$21),"00")&amp;":"&amp;TEXT(MINUTE(הגדרות!$C$21),"00"))</f>
-        <v>הדרכה 09:00–12:30</v>
+        <v/>
       </c>
       <c r="E23" s="41" t="s">
         <v>83</v>
       </c>
-      <c r="F23" s="42" t="n">
+      <c r="F23" s="42" t="str">
         <f aca="false">IF(B23="","",IF(E23="לא",0,הגדרות!$C$22))</f>
-        <v>3.5</v>
-      </c>
-      <c r="G23" s="43" t="n">
+        <v/>
+      </c>
+      <c r="G23" s="43" t="str">
         <f aca="false">IF(B23="","",F23*הגדרות!$C$24)</f>
-        <v>175</v>
+        <v/>
       </c>
       <c r="H23" s="44"/>
       <c r="I23" s="45"/>
-      <c r="K23" s="27" t="n">
+      <c r="K23" s="27" t="str">
         <f aca="false">IF(B23="","",B23+MIN(MOD(הגדרות!$D$18-WEEKDAY(B23)-1,7)+1,MOD(הגדרות!$D$19-WEEKDAY(B23)-1,7)+1))</f>
-        <v>46509</v>
+        <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11988,7 +12871,7 @@
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="38" t="n">
         <f aca="false">COUNT($B$15:$B$24)+1</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B25" s="46"/>
       <c r="C25" s="38" t="str">
@@ -12023,11 +12906,11 @@
       <c r="E26" s="47"/>
       <c r="F26" s="48" t="n">
         <f aca="false">SUM(F15:F25)</f>
-        <v>32.5</v>
+        <v>29</v>
       </c>
       <c r="G26" s="49" t="n">
         <f aca="false">SUM(G15:G25)</f>
-        <v>1625</v>
+        <v>1450</v>
       </c>
       <c r="H26" s="47"/>
       <c r="I26" s="49" t="n">
@@ -12049,7 +12932,7 @@
       <c r="H28" s="40"/>
       <c r="I28" s="42" t="n">
         <f aca="false">F26</f>
-        <v>32.5</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12063,13 +12946,13 @@
       <c r="E29" s="51"/>
       <c r="F29" s="40" t="str">
         <f aca="false">"הדרכת שיקום ("&amp;TEXT(F26,"0.0")&amp;" שעות × "&amp;הגדרות!$C$24&amp;" ₪)"</f>
-        <v>הדרכת שיקום (32.5 שעות × 50 ₪)</v>
+        <v>הדרכת שיקום (29.0 שעות × 50 ₪)</v>
       </c>
       <c r="G29" s="40"/>
       <c r="H29" s="40"/>
       <c r="I29" s="43" t="n">
         <f aca="false">G26</f>
-        <v>1625</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12107,7 +12990,7 @@
       <c r="H31" s="52"/>
       <c r="I31" s="53" t="n">
         <f aca="false">I29+I30</f>
-        <v>1625</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12127,7 +13010,7 @@
       <c r="H32" s="40"/>
       <c r="I32" s="43" t="n">
         <f aca="false">ROUND(I31*הגדרות!$C$25,2)</f>
-        <v>292.5</v>
+        <v>261</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12138,7 +13021,7 @@
       <c r="H33" s="54"/>
       <c r="I33" s="55" t="n">
         <f aca="false">I31+I32</f>
-        <v>1917.5</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Hosen: flat 600 fee for cancellation without notice; update business name
A meeting cancelled less than 48 hours ahead is now billed a flat
cancellation fee (600, set in settings) with no wood budget, shown as its
own line in the summary and as a term in the printed cancellation
conditions. Business name updated in both workbooks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GcyaTAwk1vz9KMfGvL4b7o
</commit_message>
<xml_diff>
--- a/quotes/הצעת-מחיר-חודשית-חוות-רום.xlsx
+++ b/quotes/הצעת-מחיר-חודשית-חוות-רום.xlsx
@@ -906,7 +906,7 @@
     <t xml:space="preserve">שם העסק</t>
   </si>
   <si>
-    <t xml:space="preserve">הנגרייה</t>
+    <t xml:space="preserve">הנגרייה השיקומית בחוות רום</t>
   </si>
   <si>
     <t xml:space="preserve">ראשון</t>
@@ -2147,7 +2147,7 @@
       <c r="B5" s="30"/>
       <c r="C5" s="31" t="str">
         <f aca="false">הגדרות!$C$5</f>
-        <v>הנגרייה</v>
+        <v>הנגרייה השיקומית בחוות רום</v>
       </c>
       <c r="D5" s="31"/>
       <c r="F5" s="30" t="s">
@@ -2979,7 +2979,7 @@
       <c r="B5" s="30"/>
       <c r="C5" s="31" t="str">
         <f aca="false">הגדרות!$C$5</f>
-        <v>הנגרייה</v>
+        <v>הנגרייה השיקומית בחוות רום</v>
       </c>
       <c r="D5" s="31"/>
       <c r="F5" s="30" t="s">
@@ -3811,7 +3811,7 @@
       <c r="B5" s="30"/>
       <c r="C5" s="31" t="str">
         <f aca="false">הגדרות!$C$5</f>
-        <v>הנגרייה</v>
+        <v>הנגרייה השיקומית בחוות רום</v>
       </c>
       <c r="D5" s="31"/>
       <c r="F5" s="30" t="s">
@@ -4643,7 +4643,7 @@
       <c r="B5" s="30"/>
       <c r="C5" s="31" t="str">
         <f aca="false">הגדרות!$C$5</f>
-        <v>הנגרייה</v>
+        <v>הנגרייה השיקומית בחוות רום</v>
       </c>
       <c r="D5" s="31"/>
       <c r="F5" s="30" t="s">
@@ -5475,7 +5475,7 @@
       <c r="B5" s="30"/>
       <c r="C5" s="31" t="str">
         <f aca="false">הגדרות!$C$5</f>
-        <v>הנגרייה</v>
+        <v>הנגרייה השיקומית בחוות רום</v>
       </c>
       <c r="D5" s="31"/>
       <c r="F5" s="30" t="s">
@@ -6307,7 +6307,7 @@
       <c r="B5" s="30"/>
       <c r="C5" s="31" t="str">
         <f aca="false">הגדרות!$C$5</f>
-        <v>הנגרייה</v>
+        <v>הנגרייה השיקומית בחוות רום</v>
       </c>
       <c r="D5" s="31"/>
       <c r="F5" s="30" t="s">
@@ -7404,7 +7404,7 @@
       <c r="B5" s="30"/>
       <c r="C5" s="31" t="str">
         <f aca="false">הגדרות!$C$5</f>
-        <v>הנגרייה</v>
+        <v>הנגרייה השיקומית בחוות רום</v>
       </c>
       <c r="D5" s="31"/>
       <c r="F5" s="30" t="s">
@@ -8236,7 +8236,7 @@
       <c r="B5" s="30"/>
       <c r="C5" s="31" t="str">
         <f aca="false">הגדרות!$C$5</f>
-        <v>הנגרייה</v>
+        <v>הנגרייה השיקומית בחוות רום</v>
       </c>
       <c r="D5" s="31"/>
       <c r="F5" s="30" t="s">
@@ -9068,7 +9068,7 @@
       <c r="B5" s="30"/>
       <c r="C5" s="31" t="str">
         <f aca="false">הגדרות!$C$5</f>
-        <v>הנגרייה</v>
+        <v>הנגרייה השיקומית בחוות רום</v>
       </c>
       <c r="D5" s="31"/>
       <c r="F5" s="30" t="s">
@@ -9900,7 +9900,7 @@
       <c r="B5" s="30"/>
       <c r="C5" s="31" t="str">
         <f aca="false">הגדרות!$C$5</f>
-        <v>הנגרייה</v>
+        <v>הנגרייה השיקומית בחוות רום</v>
       </c>
       <c r="D5" s="31"/>
       <c r="F5" s="30" t="s">
@@ -10732,7 +10732,7 @@
       <c r="B5" s="30"/>
       <c r="C5" s="31" t="str">
         <f aca="false">הגדרות!$C$5</f>
-        <v>הנגרייה</v>
+        <v>הנגרייה השיקומית בחוות רום</v>
       </c>
       <c r="D5" s="31"/>
       <c r="F5" s="30" t="s">
@@ -11564,7 +11564,7 @@
       <c r="B5" s="30"/>
       <c r="C5" s="31" t="str">
         <f aca="false">הגדרות!$C$5</f>
-        <v>הנגרייה</v>
+        <v>הנגרייה השיקומית בחוות רום</v>
       </c>
       <c r="D5" s="31"/>
       <c r="F5" s="30" t="s">
@@ -12396,7 +12396,7 @@
       <c r="B5" s="30"/>
       <c r="C5" s="31" t="str">
         <f aca="false">הגדרות!$C$5</f>
-        <v>הנגרייה</v>
+        <v>הנגרייה השיקומית בחוות רום</v>
       </c>
       <c r="D5" s="31"/>
       <c r="F5" s="30" t="s">

</xml_diff>